<commit_message>
Explainability Methods Utilized throughout the papers
</commit_message>
<xml_diff>
--- a/Phase-1-Literature-Review/Explainability/Papers/Explainability-Utilised-Methods.xlsx
+++ b/Phase-1-Literature-Review/Explainability/Papers/Explainability-Utilised-Methods.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>Authors</t>
   </si>
@@ -19,15 +19,6 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Publication</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Publisher</t>
-  </si>
-  <si>
     <t>Explainability Method</t>
   </si>
   <si>
@@ -37,9 +28,6 @@
     <t>Understanding the inner workings of large language models: Interpretability and explainability</t>
   </si>
   <si>
-    <t>MZ Journal of Artificial Intelligence</t>
-  </si>
-  <si>
     <t>The paper is a survey-type review that covers attention-based explanations, gradient/saliency-based attribution methods, and model-agnostic techniques like LIME to understand LLM decisions.</t>
   </si>
   <si>
@@ -49,12 +37,6 @@
     <t>Cost, usability, credibility, fairness, accountability, transparency, and explainability framework for safe and effective large language models in medical education: Narrative review and qualitative study</t>
   </si>
   <si>
-    <t>Jmir Ai</t>
-  </si>
-  <si>
-    <t>JMIR Publications Inc., Toronto, Canada</t>
-  </si>
-  <si>
     <t>High‑level conceptual framework: treats explainability as a key enabler in LLM adoption and evaluation (CUC‑FATE), no specific algorithmic explainability method applied.</t>
   </si>
   <si>
@@ -64,12 +46,6 @@
     <t>Evaluating the Explainability of Large Language Models for Ethical Decision Making</t>
   </si>
   <si>
-    <t>2025 IEEE International Conference on Consumer Electronics (ICCE)</t>
-  </si>
-  <si>
-    <t>IEEE</t>
-  </si>
-  <si>
     <t>Justification-based explainability using prompting strategies and latent semantic analysis (LSA) to evaluate consistency of LLM-generated explanations across moral scenarios</t>
   </si>
   <si>
@@ -79,12 +55,6 @@
     <t>The Impact of Activation Patterns in the Explainability of Large Language Models–A Survey of recent advances</t>
   </si>
   <si>
-    <t>Escola Regional de Banco de Dados (ERBD)</t>
-  </si>
-  <si>
-    <t>SBC</t>
-  </si>
-  <si>
     <t>Survey of neuron activation-based explainability methods for LLMs, including neuron relevance ranking, activation visualization, mechanistic interpretability, and manipulation of activation patterns in Transformer models.</t>
   </si>
   <si>
@@ -121,9 +91,6 @@
     <t>Automatic Programming: Large Language Models and Beyond</t>
   </si>
   <si>
-    <t>ACM</t>
-  </si>
-  <si>
     <t>Discussion oriented: addresses trust/quality of LLM‑generated code and the role of program repair/assurance in automatic programming — no dedicated algorithmic LLM explainability method described.</t>
   </si>
   <si>
@@ -185,9 +152,6 @@
   </si>
   <si>
     <t>Enhancing Trust in Generative AI: Investigating Explainability of LLMs to Analyse Confusion in MOOC Discussions</t>
-  </si>
-  <si>
-    <t>Scopus</t>
   </si>
   <si>
     <t>In this pilot study, they apply a specific XAI method, namely Integrated Gradients, to analyse how an LLM identifies word‐level indicators of student confusion in MOOC forum posts. Hence the explainability method is Integrated Gradients (gradient‐based attribution) applied to LLM predictions in an educational context.</t>
@@ -210,9 +174,6 @@
     <t>Mind the XAI Gap: A Human-Centered LLM Framework for Democratizing Explainable AI</t>
   </si>
   <si>
-    <t>The 3rd World Conference on eXplainable Artificial Intelligence.</t>
-  </si>
-  <si>
     <t>LLM‑based explanation generation framework using structured prompting for human‑centred explainability (model‑agnostic, domain‑agnostic).</t>
   </si>
   <si>
@@ -221,9 +182,6 @@
   <si>
     <t xml:space="preserve">Explainable Artificial Intelligence (XAI) in the Era of Large Language Models: Applying an XAI Framework in Pediatric Ophthalmology Diagnosis using the Gemini Model
 </t>
-  </si>
-  <si>
-    <t>PubMed</t>
   </si>
   <si>
     <t>They apply a Feature‑Guided Interpretive Prompting (FGIP) framework together with the Gemini large language model on high‑fidelity eye‑tracking data (pediatric ophthalmology) and evaluate explanations using the Quantus framework which comprises metrics such as faithfulness, robustness, localisation and complexity.</t>
@@ -236,9 +194,6 @@
   <si>
     <t xml:space="preserve">Hybrid Multi-Agent GraphRAG for E-Government: Towards a Trustworthy AI Assistant
 </t>
-  </si>
-  <si>
-    <t>MDPI</t>
   </si>
   <si>
     <t>This paper uses a multi‑agent retrieval‑augmented‑generation (RAG) architecture enhanced by knowledge‑graph (GraphRAG) modules in an e‑government setting. The explainability dimension is achieved via structured retrieval plus graph‑based provenance, enabling the assistant to reference and ground responses in verifiable knowledge.</t>
@@ -260,9 +215,6 @@
   </si>
   <si>
     <t>Explainability in LLMs and the Role of Knowledge Representation and Reasoning: A Survey</t>
-  </si>
-  <si>
-    <t>ANU</t>
   </si>
   <si>
     <t>This is a survey paper focusing on how knowledge representation and reasoning techniques support explainability in large language models. It does not present a new algorithmic explainability method but reviews how knowledge‑centric methods (e.g., symbolic reasoning, knowledge graphs, chain‑of‑thought prompting) integrate with LLMs for interpretation.</t>
@@ -364,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -378,13 +330,7 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -614,10 +560,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="35.0"/>
     <col customWidth="1" min="2" max="2" width="44.75"/>
-    <col customWidth="1" min="3" max="3" width="28.5"/>
-    <col customWidth="1" min="5" max="5" width="19.75"/>
-    <col customWidth="1" min="6" max="6" width="15.5"/>
-    <col customWidth="1" min="7" max="7" width="54.88"/>
+    <col customWidth="1" min="3" max="3" width="54.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,3443 +570,3207 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3" t="s">
-        <v>19</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="3" t="s">
-        <v>24</v>
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="3" t="s">
-        <v>30</v>
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="3" t="s">
-        <v>33</v>
+        <v>22</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="3" t="s">
-        <v>37</v>
+        <v>25</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="3" t="s">
-        <v>40</v>
+        <v>28</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="3" t="s">
-        <v>43</v>
+        <v>31</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="3" t="s">
-        <v>46</v>
+        <v>34</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="3" t="s">
-        <v>49</v>
+        <v>37</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="3" t="s">
-        <v>52</v>
+        <v>40</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="3" t="s">
-        <v>55</v>
+        <v>43</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="4">
-        <v>2024.0</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="3" t="s">
-        <v>59</v>
+        <v>46</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="3" t="s">
-        <v>62</v>
+        <v>49</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="3" t="s">
-        <v>66</v>
+        <v>52</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="3" t="s">
-        <v>70</v>
+        <v>55</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="3" t="s">
-        <v>74</v>
+        <v>58</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="3" t="s">
-        <v>77</v>
+        <v>61</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="4">
-        <v>2025.0</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="3" t="s">
-        <v>96</v>
-      </c>
     </row>
     <row r="28">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="7"/>
     </row>
     <row r="29">
-      <c r="A29" s="10"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="7"/>
     </row>
     <row r="30">
-      <c r="A30" s="10"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="7"/>
     </row>
     <row r="31">
-      <c r="A31" s="10"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="7"/>
     </row>
     <row r="32">
-      <c r="A32" s="10"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="7"/>
     </row>
     <row r="33">
-      <c r="A33" s="10"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="7"/>
     </row>
     <row r="34">
-      <c r="A34" s="10"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="7"/>
     </row>
     <row r="35">
-      <c r="A35" s="10"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="7"/>
     </row>
     <row r="36">
-      <c r="A36" s="10"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="7"/>
     </row>
     <row r="37">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
     </row>
     <row r="38">
-      <c r="G38" s="9"/>
+      <c r="C38" s="7"/>
     </row>
     <row r="39">
-      <c r="G39" s="9"/>
+      <c r="C39" s="7"/>
     </row>
     <row r="40">
-      <c r="G40" s="9"/>
+      <c r="C40" s="7"/>
     </row>
     <row r="41">
-      <c r="G41" s="9"/>
+      <c r="C41" s="7"/>
     </row>
     <row r="42">
-      <c r="G42" s="9"/>
+      <c r="C42" s="7"/>
     </row>
     <row r="43">
-      <c r="G43" s="9"/>
+      <c r="C43" s="7"/>
     </row>
     <row r="44">
-      <c r="G44" s="9"/>
+      <c r="C44" s="7"/>
     </row>
     <row r="45">
-      <c r="G45" s="9"/>
+      <c r="C45" s="7"/>
     </row>
     <row r="46">
-      <c r="G46" s="9"/>
+      <c r="C46" s="7"/>
     </row>
     <row r="47">
-      <c r="G47" s="9"/>
+      <c r="C47" s="7"/>
     </row>
     <row r="48">
-      <c r="G48" s="9"/>
+      <c r="C48" s="7"/>
     </row>
     <row r="49">
-      <c r="G49" s="9"/>
+      <c r="C49" s="7"/>
     </row>
     <row r="50">
-      <c r="G50" s="9"/>
+      <c r="C50" s="7"/>
     </row>
     <row r="51">
-      <c r="G51" s="9"/>
+      <c r="C51" s="7"/>
     </row>
     <row r="52">
-      <c r="G52" s="9"/>
+      <c r="C52" s="7"/>
     </row>
     <row r="53">
-      <c r="G53" s="9"/>
+      <c r="C53" s="7"/>
     </row>
     <row r="54">
-      <c r="G54" s="9"/>
+      <c r="C54" s="7"/>
     </row>
     <row r="55">
-      <c r="G55" s="9"/>
+      <c r="C55" s="7"/>
     </row>
     <row r="56">
-      <c r="G56" s="9"/>
+      <c r="C56" s="7"/>
     </row>
     <row r="57">
-      <c r="G57" s="9"/>
+      <c r="C57" s="7"/>
     </row>
     <row r="58">
-      <c r="G58" s="9"/>
+      <c r="C58" s="7"/>
     </row>
     <row r="59">
-      <c r="G59" s="9"/>
+      <c r="C59" s="7"/>
     </row>
     <row r="60">
-      <c r="G60" s="9"/>
+      <c r="C60" s="7"/>
     </row>
     <row r="61">
-      <c r="G61" s="9"/>
+      <c r="C61" s="7"/>
     </row>
     <row r="62">
-      <c r="G62" s="9"/>
+      <c r="C62" s="7"/>
     </row>
     <row r="63">
-      <c r="G63" s="9"/>
+      <c r="C63" s="7"/>
     </row>
     <row r="64">
-      <c r="G64" s="9"/>
+      <c r="C64" s="7"/>
     </row>
     <row r="65">
-      <c r="G65" s="9"/>
+      <c r="C65" s="7"/>
     </row>
     <row r="66">
-      <c r="G66" s="9"/>
+      <c r="C66" s="7"/>
     </row>
     <row r="67">
-      <c r="G67" s="9"/>
+      <c r="C67" s="7"/>
     </row>
     <row r="68">
-      <c r="G68" s="9"/>
+      <c r="C68" s="7"/>
     </row>
     <row r="69">
-      <c r="G69" s="9"/>
+      <c r="C69" s="7"/>
     </row>
     <row r="70">
-      <c r="G70" s="9"/>
+      <c r="C70" s="7"/>
     </row>
     <row r="71">
-      <c r="G71" s="9"/>
+      <c r="C71" s="7"/>
     </row>
     <row r="72">
-      <c r="G72" s="9"/>
+      <c r="C72" s="7"/>
     </row>
     <row r="73">
-      <c r="G73" s="9"/>
+      <c r="C73" s="7"/>
     </row>
     <row r="74">
-      <c r="G74" s="9"/>
+      <c r="C74" s="7"/>
     </row>
     <row r="75">
-      <c r="G75" s="9"/>
+      <c r="C75" s="7"/>
     </row>
     <row r="76">
-      <c r="G76" s="9"/>
+      <c r="C76" s="7"/>
     </row>
     <row r="77">
-      <c r="G77" s="9"/>
+      <c r="C77" s="7"/>
     </row>
     <row r="78">
-      <c r="G78" s="9"/>
+      <c r="C78" s="7"/>
     </row>
     <row r="79">
-      <c r="G79" s="9"/>
+      <c r="C79" s="7"/>
     </row>
     <row r="80">
-      <c r="G80" s="9"/>
+      <c r="C80" s="7"/>
     </row>
     <row r="81">
-      <c r="G81" s="9"/>
+      <c r="C81" s="7"/>
     </row>
     <row r="82">
-      <c r="G82" s="9"/>
+      <c r="C82" s="7"/>
     </row>
     <row r="83">
-      <c r="G83" s="9"/>
+      <c r="C83" s="7"/>
     </row>
     <row r="84">
-      <c r="G84" s="9"/>
+      <c r="C84" s="7"/>
     </row>
     <row r="85">
-      <c r="G85" s="9"/>
+      <c r="C85" s="7"/>
     </row>
     <row r="86">
-      <c r="G86" s="9"/>
+      <c r="C86" s="7"/>
     </row>
     <row r="87">
-      <c r="G87" s="9"/>
+      <c r="C87" s="7"/>
     </row>
     <row r="88">
-      <c r="G88" s="9"/>
+      <c r="C88" s="7"/>
     </row>
     <row r="89">
-      <c r="G89" s="9"/>
+      <c r="C89" s="7"/>
     </row>
     <row r="90">
-      <c r="G90" s="9"/>
+      <c r="C90" s="7"/>
     </row>
     <row r="91">
-      <c r="G91" s="9"/>
+      <c r="C91" s="7"/>
     </row>
     <row r="92">
-      <c r="G92" s="9"/>
+      <c r="C92" s="7"/>
     </row>
     <row r="93">
-      <c r="G93" s="9"/>
+      <c r="C93" s="7"/>
     </row>
     <row r="94">
-      <c r="G94" s="9"/>
+      <c r="C94" s="7"/>
     </row>
     <row r="95">
-      <c r="G95" s="9"/>
+      <c r="C95" s="7"/>
     </row>
     <row r="96">
-      <c r="G96" s="9"/>
+      <c r="C96" s="7"/>
     </row>
     <row r="97">
-      <c r="G97" s="9"/>
+      <c r="C97" s="7"/>
     </row>
     <row r="98">
-      <c r="G98" s="9"/>
+      <c r="C98" s="7"/>
     </row>
     <row r="99">
-      <c r="G99" s="9"/>
+      <c r="C99" s="7"/>
     </row>
     <row r="100">
-      <c r="G100" s="9"/>
+      <c r="C100" s="7"/>
     </row>
     <row r="101">
-      <c r="G101" s="9"/>
+      <c r="C101" s="7"/>
     </row>
     <row r="102">
-      <c r="G102" s="9"/>
+      <c r="C102" s="7"/>
     </row>
     <row r="103">
-      <c r="G103" s="9"/>
+      <c r="C103" s="7"/>
     </row>
     <row r="104">
-      <c r="G104" s="9"/>
+      <c r="C104" s="7"/>
     </row>
     <row r="105">
-      <c r="G105" s="9"/>
+      <c r="C105" s="7"/>
     </row>
     <row r="106">
-      <c r="G106" s="9"/>
+      <c r="C106" s="7"/>
     </row>
     <row r="107">
-      <c r="G107" s="9"/>
+      <c r="C107" s="7"/>
     </row>
     <row r="108">
-      <c r="G108" s="9"/>
+      <c r="C108" s="7"/>
     </row>
     <row r="109">
-      <c r="G109" s="9"/>
+      <c r="C109" s="7"/>
     </row>
     <row r="110">
-      <c r="G110" s="9"/>
+      <c r="C110" s="7"/>
     </row>
     <row r="111">
-      <c r="G111" s="9"/>
+      <c r="C111" s="7"/>
     </row>
     <row r="112">
-      <c r="G112" s="9"/>
+      <c r="C112" s="7"/>
     </row>
     <row r="113">
-      <c r="G113" s="9"/>
+      <c r="C113" s="7"/>
     </row>
     <row r="114">
-      <c r="G114" s="9"/>
+      <c r="C114" s="7"/>
     </row>
     <row r="115">
-      <c r="G115" s="9"/>
+      <c r="C115" s="7"/>
     </row>
     <row r="116">
-      <c r="G116" s="9"/>
+      <c r="C116" s="7"/>
     </row>
     <row r="117">
-      <c r="G117" s="9"/>
+      <c r="C117" s="7"/>
     </row>
     <row r="118">
-      <c r="G118" s="9"/>
+      <c r="C118" s="7"/>
     </row>
     <row r="119">
-      <c r="G119" s="9"/>
+      <c r="C119" s="7"/>
     </row>
     <row r="120">
-      <c r="G120" s="9"/>
+      <c r="C120" s="7"/>
     </row>
     <row r="121">
-      <c r="G121" s="9"/>
+      <c r="C121" s="7"/>
     </row>
     <row r="122">
-      <c r="G122" s="9"/>
+      <c r="C122" s="7"/>
     </row>
     <row r="123">
-      <c r="G123" s="9"/>
+      <c r="C123" s="7"/>
     </row>
     <row r="124">
-      <c r="G124" s="9"/>
+      <c r="C124" s="7"/>
     </row>
     <row r="125">
-      <c r="G125" s="9"/>
+      <c r="C125" s="7"/>
     </row>
     <row r="126">
-      <c r="G126" s="9"/>
+      <c r="C126" s="7"/>
     </row>
     <row r="127">
-      <c r="G127" s="9"/>
+      <c r="C127" s="7"/>
     </row>
     <row r="128">
-      <c r="G128" s="9"/>
+      <c r="C128" s="7"/>
     </row>
     <row r="129">
-      <c r="G129" s="9"/>
+      <c r="C129" s="7"/>
     </row>
     <row r="130">
-      <c r="G130" s="9"/>
+      <c r="C130" s="7"/>
     </row>
     <row r="131">
-      <c r="G131" s="9"/>
+      <c r="C131" s="7"/>
     </row>
     <row r="132">
-      <c r="G132" s="9"/>
+      <c r="C132" s="7"/>
     </row>
     <row r="133">
-      <c r="G133" s="9"/>
+      <c r="C133" s="7"/>
     </row>
     <row r="134">
-      <c r="G134" s="9"/>
+      <c r="C134" s="7"/>
     </row>
     <row r="135">
-      <c r="G135" s="9"/>
+      <c r="C135" s="7"/>
     </row>
     <row r="136">
-      <c r="G136" s="9"/>
+      <c r="C136" s="7"/>
     </row>
     <row r="137">
-      <c r="G137" s="9"/>
+      <c r="C137" s="7"/>
     </row>
     <row r="138">
-      <c r="G138" s="9"/>
+      <c r="C138" s="7"/>
     </row>
     <row r="139">
-      <c r="G139" s="9"/>
+      <c r="C139" s="7"/>
     </row>
     <row r="140">
-      <c r="G140" s="9"/>
+      <c r="C140" s="7"/>
     </row>
     <row r="141">
-      <c r="G141" s="9"/>
+      <c r="C141" s="7"/>
     </row>
     <row r="142">
-      <c r="G142" s="9"/>
+      <c r="C142" s="7"/>
     </row>
     <row r="143">
-      <c r="G143" s="9"/>
+      <c r="C143" s="7"/>
     </row>
     <row r="144">
-      <c r="G144" s="9"/>
+      <c r="C144" s="7"/>
     </row>
     <row r="145">
-      <c r="G145" s="9"/>
+      <c r="C145" s="7"/>
     </row>
     <row r="146">
-      <c r="G146" s="9"/>
+      <c r="C146" s="7"/>
     </row>
     <row r="147">
-      <c r="G147" s="9"/>
+      <c r="C147" s="7"/>
     </row>
     <row r="148">
-      <c r="G148" s="9"/>
+      <c r="C148" s="7"/>
     </row>
     <row r="149">
-      <c r="G149" s="9"/>
+      <c r="C149" s="7"/>
     </row>
     <row r="150">
-      <c r="G150" s="9"/>
+      <c r="C150" s="7"/>
     </row>
     <row r="151">
-      <c r="G151" s="9"/>
+      <c r="C151" s="7"/>
     </row>
     <row r="152">
-      <c r="G152" s="9"/>
+      <c r="C152" s="7"/>
     </row>
     <row r="153">
-      <c r="G153" s="9"/>
+      <c r="C153" s="7"/>
     </row>
     <row r="154">
-      <c r="G154" s="9"/>
+      <c r="C154" s="7"/>
     </row>
     <row r="155">
-      <c r="G155" s="9"/>
+      <c r="C155" s="7"/>
     </row>
     <row r="156">
-      <c r="G156" s="9"/>
+      <c r="C156" s="7"/>
     </row>
     <row r="157">
-      <c r="G157" s="9"/>
+      <c r="C157" s="7"/>
     </row>
     <row r="158">
-      <c r="G158" s="9"/>
+      <c r="C158" s="7"/>
     </row>
     <row r="159">
-      <c r="G159" s="9"/>
+      <c r="C159" s="7"/>
     </row>
     <row r="160">
-      <c r="G160" s="9"/>
+      <c r="C160" s="7"/>
     </row>
     <row r="161">
-      <c r="G161" s="9"/>
+      <c r="C161" s="7"/>
     </row>
     <row r="162">
-      <c r="G162" s="9"/>
+      <c r="C162" s="7"/>
     </row>
     <row r="163">
-      <c r="G163" s="9"/>
+      <c r="C163" s="7"/>
     </row>
     <row r="164">
-      <c r="G164" s="9"/>
+      <c r="C164" s="7"/>
     </row>
     <row r="165">
-      <c r="G165" s="9"/>
+      <c r="C165" s="7"/>
     </row>
     <row r="166">
-      <c r="G166" s="9"/>
+      <c r="C166" s="7"/>
     </row>
     <row r="167">
-      <c r="G167" s="9"/>
+      <c r="C167" s="7"/>
     </row>
     <row r="168">
-      <c r="G168" s="9"/>
+      <c r="C168" s="7"/>
     </row>
     <row r="169">
-      <c r="G169" s="9"/>
+      <c r="C169" s="7"/>
     </row>
     <row r="170">
-      <c r="G170" s="9"/>
+      <c r="C170" s="7"/>
     </row>
     <row r="171">
-      <c r="G171" s="9"/>
+      <c r="C171" s="7"/>
     </row>
     <row r="172">
-      <c r="G172" s="9"/>
+      <c r="C172" s="7"/>
     </row>
     <row r="173">
-      <c r="G173" s="9"/>
+      <c r="C173" s="7"/>
     </row>
     <row r="174">
-      <c r="G174" s="9"/>
+      <c r="C174" s="7"/>
     </row>
     <row r="175">
-      <c r="G175" s="9"/>
+      <c r="C175" s="7"/>
     </row>
     <row r="176">
-      <c r="G176" s="9"/>
+      <c r="C176" s="7"/>
     </row>
     <row r="177">
-      <c r="G177" s="9"/>
+      <c r="C177" s="7"/>
     </row>
     <row r="178">
-      <c r="G178" s="9"/>
+      <c r="C178" s="7"/>
     </row>
     <row r="179">
-      <c r="G179" s="9"/>
+      <c r="C179" s="7"/>
     </row>
     <row r="180">
-      <c r="G180" s="9"/>
+      <c r="C180" s="7"/>
     </row>
     <row r="181">
-      <c r="G181" s="9"/>
+      <c r="C181" s="7"/>
     </row>
     <row r="182">
-      <c r="G182" s="9"/>
+      <c r="C182" s="7"/>
     </row>
     <row r="183">
-      <c r="G183" s="9"/>
+      <c r="C183" s="7"/>
     </row>
     <row r="184">
-      <c r="G184" s="9"/>
+      <c r="C184" s="7"/>
     </row>
     <row r="185">
-      <c r="G185" s="9"/>
+      <c r="C185" s="7"/>
     </row>
     <row r="186">
-      <c r="G186" s="9"/>
+      <c r="C186" s="7"/>
     </row>
     <row r="187">
-      <c r="G187" s="9"/>
+      <c r="C187" s="7"/>
     </row>
     <row r="188">
-      <c r="G188" s="9"/>
+      <c r="C188" s="7"/>
     </row>
     <row r="189">
-      <c r="G189" s="9"/>
+      <c r="C189" s="7"/>
     </row>
     <row r="190">
-      <c r="G190" s="9"/>
+      <c r="C190" s="7"/>
     </row>
     <row r="191">
-      <c r="G191" s="9"/>
+      <c r="C191" s="7"/>
     </row>
     <row r="192">
-      <c r="G192" s="9"/>
+      <c r="C192" s="7"/>
     </row>
     <row r="193">
-      <c r="G193" s="9"/>
+      <c r="C193" s="7"/>
     </row>
     <row r="194">
-      <c r="G194" s="9"/>
+      <c r="C194" s="7"/>
     </row>
     <row r="195">
-      <c r="G195" s="9"/>
+      <c r="C195" s="7"/>
     </row>
     <row r="196">
-      <c r="G196" s="9"/>
+      <c r="C196" s="7"/>
     </row>
     <row r="197">
-      <c r="G197" s="9"/>
+      <c r="C197" s="7"/>
     </row>
     <row r="198">
-      <c r="G198" s="9"/>
+      <c r="C198" s="7"/>
     </row>
     <row r="199">
-      <c r="G199" s="9"/>
+      <c r="C199" s="7"/>
     </row>
     <row r="200">
-      <c r="G200" s="9"/>
+      <c r="C200" s="7"/>
     </row>
     <row r="201">
-      <c r="G201" s="9"/>
+      <c r="C201" s="7"/>
     </row>
     <row r="202">
-      <c r="G202" s="9"/>
+      <c r="C202" s="7"/>
     </row>
     <row r="203">
-      <c r="G203" s="9"/>
+      <c r="C203" s="7"/>
     </row>
     <row r="204">
-      <c r="G204" s="9"/>
+      <c r="C204" s="7"/>
     </row>
     <row r="205">
-      <c r="G205" s="9"/>
+      <c r="C205" s="7"/>
     </row>
     <row r="206">
-      <c r="G206" s="9"/>
+      <c r="C206" s="7"/>
     </row>
     <row r="207">
-      <c r="G207" s="9"/>
+      <c r="C207" s="7"/>
     </row>
     <row r="208">
-      <c r="G208" s="9"/>
+      <c r="C208" s="7"/>
     </row>
     <row r="209">
-      <c r="G209" s="9"/>
+      <c r="C209" s="7"/>
     </row>
     <row r="210">
-      <c r="G210" s="9"/>
+      <c r="C210" s="7"/>
     </row>
     <row r="211">
-      <c r="G211" s="9"/>
+      <c r="C211" s="7"/>
     </row>
     <row r="212">
-      <c r="G212" s="9"/>
+      <c r="C212" s="7"/>
     </row>
     <row r="213">
-      <c r="G213" s="9"/>
+      <c r="C213" s="7"/>
     </row>
     <row r="214">
-      <c r="G214" s="9"/>
+      <c r="C214" s="7"/>
     </row>
     <row r="215">
-      <c r="G215" s="9"/>
+      <c r="C215" s="7"/>
     </row>
     <row r="216">
-      <c r="G216" s="9"/>
+      <c r="C216" s="7"/>
     </row>
     <row r="217">
-      <c r="G217" s="9"/>
+      <c r="C217" s="7"/>
     </row>
     <row r="218">
-      <c r="G218" s="9"/>
+      <c r="C218" s="7"/>
     </row>
     <row r="219">
-      <c r="G219" s="9"/>
+      <c r="C219" s="7"/>
     </row>
     <row r="220">
-      <c r="G220" s="9"/>
+      <c r="C220" s="7"/>
     </row>
     <row r="221">
-      <c r="G221" s="9"/>
+      <c r="C221" s="7"/>
     </row>
     <row r="222">
-      <c r="G222" s="9"/>
+      <c r="C222" s="7"/>
     </row>
     <row r="223">
-      <c r="G223" s="9"/>
+      <c r="C223" s="7"/>
     </row>
     <row r="224">
-      <c r="G224" s="9"/>
+      <c r="C224" s="7"/>
     </row>
     <row r="225">
-      <c r="G225" s="9"/>
+      <c r="C225" s="7"/>
     </row>
     <row r="226">
-      <c r="G226" s="9"/>
+      <c r="C226" s="7"/>
     </row>
     <row r="227">
-      <c r="G227" s="9"/>
+      <c r="C227" s="7"/>
     </row>
     <row r="228">
-      <c r="G228" s="9"/>
+      <c r="C228" s="7"/>
     </row>
     <row r="229">
-      <c r="G229" s="9"/>
+      <c r="C229" s="7"/>
     </row>
     <row r="230">
-      <c r="G230" s="9"/>
+      <c r="C230" s="7"/>
     </row>
     <row r="231">
-      <c r="G231" s="9"/>
+      <c r="C231" s="7"/>
     </row>
     <row r="232">
-      <c r="G232" s="9"/>
+      <c r="C232" s="7"/>
     </row>
     <row r="233">
-      <c r="G233" s="9"/>
+      <c r="C233" s="7"/>
     </row>
     <row r="234">
-      <c r="G234" s="9"/>
+      <c r="C234" s="7"/>
     </row>
     <row r="235">
-      <c r="G235" s="9"/>
+      <c r="C235" s="7"/>
     </row>
     <row r="236">
-      <c r="G236" s="9"/>
+      <c r="C236" s="7"/>
     </row>
     <row r="237">
-      <c r="G237" s="9"/>
+      <c r="C237" s="7"/>
     </row>
     <row r="238">
-      <c r="G238" s="9"/>
+      <c r="C238" s="7"/>
     </row>
     <row r="239">
-      <c r="G239" s="9"/>
+      <c r="C239" s="7"/>
     </row>
     <row r="240">
-      <c r="G240" s="9"/>
+      <c r="C240" s="7"/>
     </row>
     <row r="241">
-      <c r="G241" s="9"/>
+      <c r="C241" s="7"/>
     </row>
     <row r="242">
-      <c r="G242" s="9"/>
+      <c r="C242" s="7"/>
     </row>
     <row r="243">
-      <c r="G243" s="9"/>
+      <c r="C243" s="7"/>
     </row>
     <row r="244">
-      <c r="G244" s="9"/>
+      <c r="C244" s="7"/>
     </row>
     <row r="245">
-      <c r="G245" s="9"/>
+      <c r="C245" s="7"/>
     </row>
     <row r="246">
-      <c r="G246" s="9"/>
+      <c r="C246" s="7"/>
     </row>
     <row r="247">
-      <c r="G247" s="9"/>
+      <c r="C247" s="7"/>
     </row>
     <row r="248">
-      <c r="G248" s="9"/>
+      <c r="C248" s="7"/>
     </row>
     <row r="249">
-      <c r="G249" s="9"/>
+      <c r="C249" s="7"/>
     </row>
     <row r="250">
-      <c r="G250" s="9"/>
+      <c r="C250" s="7"/>
     </row>
     <row r="251">
-      <c r="G251" s="9"/>
+      <c r="C251" s="7"/>
     </row>
     <row r="252">
-      <c r="G252" s="9"/>
+      <c r="C252" s="7"/>
     </row>
     <row r="253">
-      <c r="G253" s="9"/>
+      <c r="C253" s="7"/>
     </row>
     <row r="254">
-      <c r="G254" s="9"/>
+      <c r="C254" s="7"/>
     </row>
     <row r="255">
-      <c r="G255" s="9"/>
+      <c r="C255" s="7"/>
     </row>
     <row r="256">
-      <c r="G256" s="9"/>
+      <c r="C256" s="7"/>
     </row>
     <row r="257">
-      <c r="G257" s="9"/>
+      <c r="C257" s="7"/>
     </row>
     <row r="258">
-      <c r="G258" s="9"/>
+      <c r="C258" s="7"/>
     </row>
     <row r="259">
-      <c r="G259" s="9"/>
+      <c r="C259" s="7"/>
     </row>
     <row r="260">
-      <c r="G260" s="9"/>
+      <c r="C260" s="7"/>
     </row>
     <row r="261">
-      <c r="G261" s="9"/>
+      <c r="C261" s="7"/>
     </row>
     <row r="262">
-      <c r="G262" s="9"/>
+      <c r="C262" s="7"/>
     </row>
     <row r="263">
-      <c r="G263" s="9"/>
+      <c r="C263" s="7"/>
     </row>
     <row r="264">
-      <c r="G264" s="9"/>
+      <c r="C264" s="7"/>
     </row>
     <row r="265">
-      <c r="G265" s="9"/>
+      <c r="C265" s="7"/>
     </row>
     <row r="266">
-      <c r="G266" s="9"/>
+      <c r="C266" s="7"/>
     </row>
     <row r="267">
-      <c r="G267" s="9"/>
+      <c r="C267" s="7"/>
     </row>
     <row r="268">
-      <c r="G268" s="9"/>
+      <c r="C268" s="7"/>
     </row>
     <row r="269">
-      <c r="G269" s="9"/>
+      <c r="C269" s="7"/>
     </row>
     <row r="270">
-      <c r="G270" s="9"/>
+      <c r="C270" s="7"/>
     </row>
     <row r="271">
-      <c r="G271" s="9"/>
+      <c r="C271" s="7"/>
     </row>
     <row r="272">
-      <c r="G272" s="9"/>
+      <c r="C272" s="7"/>
     </row>
     <row r="273">
-      <c r="G273" s="9"/>
+      <c r="C273" s="7"/>
     </row>
     <row r="274">
-      <c r="G274" s="9"/>
+      <c r="C274" s="7"/>
     </row>
     <row r="275">
-      <c r="G275" s="9"/>
+      <c r="C275" s="7"/>
     </row>
     <row r="276">
-      <c r="G276" s="9"/>
+      <c r="C276" s="7"/>
     </row>
     <row r="277">
-      <c r="G277" s="9"/>
+      <c r="C277" s="7"/>
     </row>
     <row r="278">
-      <c r="G278" s="9"/>
+      <c r="C278" s="7"/>
     </row>
     <row r="279">
-      <c r="G279" s="9"/>
+      <c r="C279" s="7"/>
     </row>
     <row r="280">
-      <c r="G280" s="9"/>
+      <c r="C280" s="7"/>
     </row>
     <row r="281">
-      <c r="G281" s="9"/>
+      <c r="C281" s="7"/>
     </row>
     <row r="282">
-      <c r="G282" s="9"/>
+      <c r="C282" s="7"/>
     </row>
     <row r="283">
-      <c r="G283" s="9"/>
+      <c r="C283" s="7"/>
     </row>
     <row r="284">
-      <c r="G284" s="9"/>
+      <c r="C284" s="7"/>
     </row>
     <row r="285">
-      <c r="G285" s="9"/>
+      <c r="C285" s="7"/>
     </row>
     <row r="286">
-      <c r="G286" s="9"/>
+      <c r="C286" s="7"/>
     </row>
     <row r="287">
-      <c r="G287" s="9"/>
+      <c r="C287" s="7"/>
     </row>
     <row r="288">
-      <c r="G288" s="9"/>
+      <c r="C288" s="7"/>
     </row>
     <row r="289">
-      <c r="G289" s="9"/>
+      <c r="C289" s="7"/>
     </row>
     <row r="290">
-      <c r="G290" s="9"/>
+      <c r="C290" s="7"/>
     </row>
     <row r="291">
-      <c r="G291" s="9"/>
+      <c r="C291" s="7"/>
     </row>
     <row r="292">
-      <c r="G292" s="9"/>
+      <c r="C292" s="7"/>
     </row>
     <row r="293">
-      <c r="G293" s="9"/>
+      <c r="C293" s="7"/>
     </row>
     <row r="294">
-      <c r="G294" s="9"/>
+      <c r="C294" s="7"/>
     </row>
     <row r="295">
-      <c r="G295" s="9"/>
+      <c r="C295" s="7"/>
     </row>
     <row r="296">
-      <c r="G296" s="9"/>
+      <c r="C296" s="7"/>
     </row>
     <row r="297">
-      <c r="G297" s="9"/>
+      <c r="C297" s="7"/>
     </row>
     <row r="298">
-      <c r="G298" s="9"/>
+      <c r="C298" s="7"/>
     </row>
     <row r="299">
-      <c r="G299" s="9"/>
+      <c r="C299" s="7"/>
     </row>
     <row r="300">
-      <c r="G300" s="9"/>
+      <c r="C300" s="7"/>
     </row>
     <row r="301">
-      <c r="G301" s="9"/>
+      <c r="C301" s="7"/>
     </row>
     <row r="302">
-      <c r="G302" s="9"/>
+      <c r="C302" s="7"/>
     </row>
     <row r="303">
-      <c r="G303" s="9"/>
+      <c r="C303" s="7"/>
     </row>
     <row r="304">
-      <c r="G304" s="9"/>
+      <c r="C304" s="7"/>
     </row>
     <row r="305">
-      <c r="G305" s="9"/>
+      <c r="C305" s="7"/>
     </row>
     <row r="306">
-      <c r="G306" s="9"/>
+      <c r="C306" s="7"/>
     </row>
     <row r="307">
-      <c r="G307" s="9"/>
+      <c r="C307" s="7"/>
     </row>
     <row r="308">
-      <c r="G308" s="9"/>
+      <c r="C308" s="7"/>
     </row>
     <row r="309">
-      <c r="G309" s="9"/>
+      <c r="C309" s="7"/>
     </row>
     <row r="310">
-      <c r="G310" s="9"/>
+      <c r="C310" s="7"/>
     </row>
     <row r="311">
-      <c r="G311" s="9"/>
+      <c r="C311" s="7"/>
     </row>
     <row r="312">
-      <c r="G312" s="9"/>
+      <c r="C312" s="7"/>
     </row>
     <row r="313">
-      <c r="G313" s="9"/>
+      <c r="C313" s="7"/>
     </row>
     <row r="314">
-      <c r="G314" s="9"/>
+      <c r="C314" s="7"/>
     </row>
     <row r="315">
-      <c r="G315" s="9"/>
+      <c r="C315" s="7"/>
     </row>
     <row r="316">
-      <c r="G316" s="9"/>
+      <c r="C316" s="7"/>
     </row>
     <row r="317">
-      <c r="G317" s="9"/>
+      <c r="C317" s="7"/>
     </row>
     <row r="318">
-      <c r="G318" s="9"/>
+      <c r="C318" s="7"/>
     </row>
     <row r="319">
-      <c r="G319" s="9"/>
+      <c r="C319" s="7"/>
     </row>
     <row r="320">
-      <c r="G320" s="9"/>
+      <c r="C320" s="7"/>
     </row>
     <row r="321">
-      <c r="G321" s="9"/>
+      <c r="C321" s="7"/>
     </row>
     <row r="322">
-      <c r="G322" s="9"/>
+      <c r="C322" s="7"/>
     </row>
     <row r="323">
-      <c r="G323" s="9"/>
+      <c r="C323" s="7"/>
     </row>
     <row r="324">
-      <c r="G324" s="9"/>
+      <c r="C324" s="7"/>
     </row>
     <row r="325">
-      <c r="G325" s="9"/>
+      <c r="C325" s="7"/>
     </row>
     <row r="326">
-      <c r="G326" s="9"/>
+      <c r="C326" s="7"/>
     </row>
     <row r="327">
-      <c r="G327" s="9"/>
+      <c r="C327" s="7"/>
     </row>
     <row r="328">
-      <c r="G328" s="9"/>
+      <c r="C328" s="7"/>
     </row>
     <row r="329">
-      <c r="G329" s="9"/>
+      <c r="C329" s="7"/>
     </row>
     <row r="330">
-      <c r="G330" s="9"/>
+      <c r="C330" s="7"/>
     </row>
     <row r="331">
-      <c r="G331" s="9"/>
+      <c r="C331" s="7"/>
     </row>
     <row r="332">
-      <c r="G332" s="9"/>
+      <c r="C332" s="7"/>
     </row>
     <row r="333">
-      <c r="G333" s="9"/>
+      <c r="C333" s="7"/>
     </row>
     <row r="334">
-      <c r="G334" s="9"/>
+      <c r="C334" s="7"/>
     </row>
     <row r="335">
-      <c r="G335" s="9"/>
+      <c r="C335" s="7"/>
     </row>
     <row r="336">
-      <c r="G336" s="9"/>
+      <c r="C336" s="7"/>
     </row>
     <row r="337">
-      <c r="G337" s="9"/>
+      <c r="C337" s="7"/>
     </row>
     <row r="338">
-      <c r="G338" s="9"/>
+      <c r="C338" s="7"/>
     </row>
     <row r="339">
-      <c r="G339" s="9"/>
+      <c r="C339" s="7"/>
     </row>
     <row r="340">
-      <c r="G340" s="9"/>
+      <c r="C340" s="7"/>
     </row>
     <row r="341">
-      <c r="G341" s="9"/>
+      <c r="C341" s="7"/>
     </row>
     <row r="342">
-      <c r="G342" s="9"/>
+      <c r="C342" s="7"/>
     </row>
     <row r="343">
-      <c r="G343" s="9"/>
+      <c r="C343" s="7"/>
     </row>
     <row r="344">
-      <c r="G344" s="9"/>
+      <c r="C344" s="7"/>
     </row>
     <row r="345">
-      <c r="G345" s="9"/>
+      <c r="C345" s="7"/>
     </row>
     <row r="346">
-      <c r="G346" s="9"/>
+      <c r="C346" s="7"/>
     </row>
     <row r="347">
-      <c r="G347" s="9"/>
+      <c r="C347" s="7"/>
     </row>
     <row r="348">
-      <c r="G348" s="9"/>
+      <c r="C348" s="7"/>
     </row>
     <row r="349">
-      <c r="G349" s="9"/>
+      <c r="C349" s="7"/>
     </row>
     <row r="350">
-      <c r="G350" s="9"/>
+      <c r="C350" s="7"/>
     </row>
     <row r="351">
-      <c r="G351" s="9"/>
+      <c r="C351" s="7"/>
     </row>
     <row r="352">
-      <c r="G352" s="9"/>
+      <c r="C352" s="7"/>
     </row>
     <row r="353">
-      <c r="G353" s="9"/>
+      <c r="C353" s="7"/>
     </row>
     <row r="354">
-      <c r="G354" s="9"/>
+      <c r="C354" s="7"/>
     </row>
     <row r="355">
-      <c r="G355" s="9"/>
+      <c r="C355" s="7"/>
     </row>
     <row r="356">
-      <c r="G356" s="9"/>
+      <c r="C356" s="7"/>
     </row>
     <row r="357">
-      <c r="G357" s="9"/>
+      <c r="C357" s="7"/>
     </row>
     <row r="358">
-      <c r="G358" s="9"/>
+      <c r="C358" s="7"/>
     </row>
     <row r="359">
-      <c r="G359" s="9"/>
+      <c r="C359" s="7"/>
     </row>
     <row r="360">
-      <c r="G360" s="9"/>
+      <c r="C360" s="7"/>
     </row>
     <row r="361">
-      <c r="G361" s="9"/>
+      <c r="C361" s="7"/>
     </row>
     <row r="362">
-      <c r="G362" s="9"/>
+      <c r="C362" s="7"/>
     </row>
     <row r="363">
-      <c r="G363" s="9"/>
+      <c r="C363" s="7"/>
     </row>
     <row r="364">
-      <c r="G364" s="9"/>
+      <c r="C364" s="7"/>
     </row>
     <row r="365">
-      <c r="G365" s="9"/>
+      <c r="C365" s="7"/>
     </row>
     <row r="366">
-      <c r="G366" s="9"/>
+      <c r="C366" s="7"/>
     </row>
     <row r="367">
-      <c r="G367" s="9"/>
+      <c r="C367" s="7"/>
     </row>
     <row r="368">
-      <c r="G368" s="9"/>
+      <c r="C368" s="7"/>
     </row>
     <row r="369">
-      <c r="G369" s="9"/>
+      <c r="C369" s="7"/>
     </row>
     <row r="370">
-      <c r="G370" s="9"/>
+      <c r="C370" s="7"/>
     </row>
     <row r="371">
-      <c r="G371" s="9"/>
+      <c r="C371" s="7"/>
     </row>
     <row r="372">
-      <c r="G372" s="9"/>
+      <c r="C372" s="7"/>
     </row>
     <row r="373">
-      <c r="G373" s="9"/>
+      <c r="C373" s="7"/>
     </row>
     <row r="374">
-      <c r="G374" s="9"/>
+      <c r="C374" s="7"/>
     </row>
     <row r="375">
-      <c r="G375" s="9"/>
+      <c r="C375" s="7"/>
     </row>
     <row r="376">
-      <c r="G376" s="9"/>
+      <c r="C376" s="7"/>
     </row>
     <row r="377">
-      <c r="G377" s="9"/>
+      <c r="C377" s="7"/>
     </row>
     <row r="378">
-      <c r="G378" s="9"/>
+      <c r="C378" s="7"/>
     </row>
     <row r="379">
-      <c r="G379" s="9"/>
+      <c r="C379" s="7"/>
     </row>
     <row r="380">
-      <c r="G380" s="9"/>
+      <c r="C380" s="7"/>
     </row>
     <row r="381">
-      <c r="G381" s="9"/>
+      <c r="C381" s="7"/>
     </row>
     <row r="382">
-      <c r="G382" s="9"/>
+      <c r="C382" s="7"/>
     </row>
     <row r="383">
-      <c r="G383" s="9"/>
+      <c r="C383" s="7"/>
     </row>
     <row r="384">
-      <c r="G384" s="9"/>
+      <c r="C384" s="7"/>
     </row>
     <row r="385">
-      <c r="G385" s="9"/>
+      <c r="C385" s="7"/>
     </row>
     <row r="386">
-      <c r="G386" s="9"/>
+      <c r="C386" s="7"/>
     </row>
     <row r="387">
-      <c r="G387" s="9"/>
+      <c r="C387" s="7"/>
     </row>
     <row r="388">
-      <c r="G388" s="9"/>
+      <c r="C388" s="7"/>
     </row>
     <row r="389">
-      <c r="G389" s="9"/>
+      <c r="C389" s="7"/>
     </row>
     <row r="390">
-      <c r="G390" s="9"/>
+      <c r="C390" s="7"/>
     </row>
     <row r="391">
-      <c r="G391" s="9"/>
+      <c r="C391" s="7"/>
     </row>
     <row r="392">
-      <c r="G392" s="9"/>
+      <c r="C392" s="7"/>
     </row>
     <row r="393">
-      <c r="G393" s="9"/>
+      <c r="C393" s="7"/>
     </row>
     <row r="394">
-      <c r="G394" s="9"/>
+      <c r="C394" s="7"/>
     </row>
     <row r="395">
-      <c r="G395" s="9"/>
+      <c r="C395" s="7"/>
     </row>
     <row r="396">
-      <c r="G396" s="9"/>
+      <c r="C396" s="7"/>
     </row>
     <row r="397">
-      <c r="G397" s="9"/>
+      <c r="C397" s="7"/>
     </row>
     <row r="398">
-      <c r="G398" s="9"/>
+      <c r="C398" s="7"/>
     </row>
     <row r="399">
-      <c r="G399" s="9"/>
+      <c r="C399" s="7"/>
     </row>
     <row r="400">
-      <c r="G400" s="9"/>
+      <c r="C400" s="7"/>
     </row>
     <row r="401">
-      <c r="G401" s="9"/>
+      <c r="C401" s="7"/>
     </row>
     <row r="402">
-      <c r="G402" s="9"/>
+      <c r="C402" s="7"/>
     </row>
     <row r="403">
-      <c r="G403" s="9"/>
+      <c r="C403" s="7"/>
     </row>
     <row r="404">
-      <c r="G404" s="9"/>
+      <c r="C404" s="7"/>
     </row>
     <row r="405">
-      <c r="G405" s="9"/>
+      <c r="C405" s="7"/>
     </row>
     <row r="406">
-      <c r="G406" s="9"/>
+      <c r="C406" s="7"/>
     </row>
     <row r="407">
-      <c r="G407" s="9"/>
+      <c r="C407" s="7"/>
     </row>
     <row r="408">
-      <c r="G408" s="9"/>
+      <c r="C408" s="7"/>
     </row>
     <row r="409">
-      <c r="G409" s="9"/>
+      <c r="C409" s="7"/>
     </row>
     <row r="410">
-      <c r="G410" s="9"/>
+      <c r="C410" s="7"/>
     </row>
     <row r="411">
-      <c r="G411" s="9"/>
+      <c r="C411" s="7"/>
     </row>
     <row r="412">
-      <c r="G412" s="9"/>
+      <c r="C412" s="7"/>
     </row>
     <row r="413">
-      <c r="G413" s="9"/>
+      <c r="C413" s="7"/>
     </row>
     <row r="414">
-      <c r="G414" s="9"/>
+      <c r="C414" s="7"/>
     </row>
     <row r="415">
-      <c r="G415" s="9"/>
+      <c r="C415" s="7"/>
     </row>
     <row r="416">
-      <c r="G416" s="9"/>
+      <c r="C416" s="7"/>
     </row>
     <row r="417">
-      <c r="G417" s="9"/>
+      <c r="C417" s="7"/>
     </row>
     <row r="418">
-      <c r="G418" s="9"/>
+      <c r="C418" s="7"/>
     </row>
     <row r="419">
-      <c r="G419" s="9"/>
+      <c r="C419" s="7"/>
     </row>
     <row r="420">
-      <c r="G420" s="9"/>
+      <c r="C420" s="7"/>
     </row>
     <row r="421">
-      <c r="G421" s="9"/>
+      <c r="C421" s="7"/>
     </row>
     <row r="422">
-      <c r="G422" s="9"/>
+      <c r="C422" s="7"/>
     </row>
     <row r="423">
-      <c r="G423" s="9"/>
+      <c r="C423" s="7"/>
     </row>
     <row r="424">
-      <c r="G424" s="9"/>
+      <c r="C424" s="7"/>
     </row>
     <row r="425">
-      <c r="G425" s="9"/>
+      <c r="C425" s="7"/>
     </row>
     <row r="426">
-      <c r="G426" s="9"/>
+      <c r="C426" s="7"/>
     </row>
     <row r="427">
-      <c r="G427" s="9"/>
+      <c r="C427" s="7"/>
     </row>
     <row r="428">
-      <c r="G428" s="9"/>
+      <c r="C428" s="7"/>
     </row>
     <row r="429">
-      <c r="G429" s="9"/>
+      <c r="C429" s="7"/>
     </row>
     <row r="430">
-      <c r="G430" s="9"/>
+      <c r="C430" s="7"/>
     </row>
     <row r="431">
-      <c r="G431" s="9"/>
+      <c r="C431" s="7"/>
     </row>
     <row r="432">
-      <c r="G432" s="9"/>
+      <c r="C432" s="7"/>
     </row>
     <row r="433">
-      <c r="G433" s="9"/>
+      <c r="C433" s="7"/>
     </row>
     <row r="434">
-      <c r="G434" s="9"/>
+      <c r="C434" s="7"/>
     </row>
     <row r="435">
-      <c r="G435" s="9"/>
+      <c r="C435" s="7"/>
     </row>
     <row r="436">
-      <c r="G436" s="9"/>
+      <c r="C436" s="7"/>
     </row>
     <row r="437">
-      <c r="G437" s="9"/>
+      <c r="C437" s="7"/>
     </row>
     <row r="438">
-      <c r="G438" s="9"/>
+      <c r="C438" s="7"/>
     </row>
     <row r="439">
-      <c r="G439" s="9"/>
+      <c r="C439" s="7"/>
     </row>
     <row r="440">
-      <c r="G440" s="9"/>
+      <c r="C440" s="7"/>
     </row>
     <row r="441">
-      <c r="G441" s="9"/>
+      <c r="C441" s="7"/>
     </row>
     <row r="442">
-      <c r="G442" s="9"/>
+      <c r="C442" s="7"/>
     </row>
     <row r="443">
-      <c r="G443" s="9"/>
+      <c r="C443" s="7"/>
     </row>
     <row r="444">
-      <c r="G444" s="9"/>
+      <c r="C444" s="7"/>
     </row>
     <row r="445">
-      <c r="G445" s="9"/>
+      <c r="C445" s="7"/>
     </row>
     <row r="446">
-      <c r="G446" s="9"/>
+      <c r="C446" s="7"/>
     </row>
     <row r="447">
-      <c r="G447" s="9"/>
+      <c r="C447" s="7"/>
     </row>
     <row r="448">
-      <c r="G448" s="9"/>
+      <c r="C448" s="7"/>
     </row>
     <row r="449">
-      <c r="G449" s="9"/>
+      <c r="C449" s="7"/>
     </row>
     <row r="450">
-      <c r="G450" s="9"/>
+      <c r="C450" s="7"/>
     </row>
     <row r="451">
-      <c r="G451" s="9"/>
+      <c r="C451" s="7"/>
     </row>
     <row r="452">
-      <c r="G452" s="9"/>
+      <c r="C452" s="7"/>
     </row>
     <row r="453">
-      <c r="G453" s="9"/>
+      <c r="C453" s="7"/>
     </row>
     <row r="454">
-      <c r="G454" s="9"/>
+      <c r="C454" s="7"/>
     </row>
     <row r="455">
-      <c r="G455" s="9"/>
+      <c r="C455" s="7"/>
     </row>
     <row r="456">
-      <c r="G456" s="9"/>
+      <c r="C456" s="7"/>
     </row>
     <row r="457">
-      <c r="G457" s="9"/>
+      <c r="C457" s="7"/>
     </row>
     <row r="458">
-      <c r="G458" s="9"/>
+      <c r="C458" s="7"/>
     </row>
     <row r="459">
-      <c r="G459" s="9"/>
+      <c r="C459" s="7"/>
     </row>
     <row r="460">
-      <c r="G460" s="9"/>
+      <c r="C460" s="7"/>
     </row>
     <row r="461">
-      <c r="G461" s="9"/>
+      <c r="C461" s="7"/>
     </row>
     <row r="462">
-      <c r="G462" s="9"/>
+      <c r="C462" s="7"/>
     </row>
     <row r="463">
-      <c r="G463" s="9"/>
+      <c r="C463" s="7"/>
     </row>
     <row r="464">
-      <c r="G464" s="9"/>
+      <c r="C464" s="7"/>
     </row>
     <row r="465">
-      <c r="G465" s="9"/>
+      <c r="C465" s="7"/>
     </row>
     <row r="466">
-      <c r="G466" s="9"/>
+      <c r="C466" s="7"/>
     </row>
     <row r="467">
-      <c r="G467" s="9"/>
+      <c r="C467" s="7"/>
     </row>
     <row r="468">
-      <c r="G468" s="9"/>
+      <c r="C468" s="7"/>
     </row>
     <row r="469">
-      <c r="G469" s="9"/>
+      <c r="C469" s="7"/>
     </row>
     <row r="470">
-      <c r="G470" s="9"/>
+      <c r="C470" s="7"/>
     </row>
     <row r="471">
-      <c r="G471" s="9"/>
+      <c r="C471" s="7"/>
     </row>
     <row r="472">
-      <c r="G472" s="9"/>
+      <c r="C472" s="7"/>
     </row>
     <row r="473">
-      <c r="G473" s="9"/>
+      <c r="C473" s="7"/>
     </row>
     <row r="474">
-      <c r="G474" s="9"/>
+      <c r="C474" s="7"/>
     </row>
     <row r="475">
-      <c r="G475" s="9"/>
+      <c r="C475" s="7"/>
     </row>
     <row r="476">
-      <c r="G476" s="9"/>
+      <c r="C476" s="7"/>
     </row>
     <row r="477">
-      <c r="G477" s="9"/>
+      <c r="C477" s="7"/>
     </row>
     <row r="478">
-      <c r="G478" s="9"/>
+      <c r="C478" s="7"/>
     </row>
     <row r="479">
-      <c r="G479" s="9"/>
+      <c r="C479" s="7"/>
     </row>
     <row r="480">
-      <c r="G480" s="9"/>
+      <c r="C480" s="7"/>
     </row>
     <row r="481">
-      <c r="G481" s="9"/>
+      <c r="C481" s="7"/>
     </row>
     <row r="482">
-      <c r="G482" s="9"/>
+      <c r="C482" s="7"/>
     </row>
     <row r="483">
-      <c r="G483" s="9"/>
+      <c r="C483" s="7"/>
     </row>
     <row r="484">
-      <c r="G484" s="9"/>
+      <c r="C484" s="7"/>
     </row>
     <row r="485">
-      <c r="G485" s="9"/>
+      <c r="C485" s="7"/>
     </row>
     <row r="486">
-      <c r="G486" s="9"/>
+      <c r="C486" s="7"/>
     </row>
     <row r="487">
-      <c r="G487" s="9"/>
+      <c r="C487" s="7"/>
     </row>
     <row r="488">
-      <c r="G488" s="9"/>
+      <c r="C488" s="7"/>
     </row>
     <row r="489">
-      <c r="G489" s="9"/>
+      <c r="C489" s="7"/>
     </row>
     <row r="490">
-      <c r="G490" s="9"/>
+      <c r="C490" s="7"/>
     </row>
     <row r="491">
-      <c r="G491" s="9"/>
+      <c r="C491" s="7"/>
     </row>
     <row r="492">
-      <c r="G492" s="9"/>
+      <c r="C492" s="7"/>
     </row>
     <row r="493">
-      <c r="G493" s="9"/>
+      <c r="C493" s="7"/>
     </row>
     <row r="494">
-      <c r="G494" s="9"/>
+      <c r="C494" s="7"/>
     </row>
     <row r="495">
-      <c r="G495" s="9"/>
+      <c r="C495" s="7"/>
     </row>
     <row r="496">
-      <c r="G496" s="9"/>
+      <c r="C496" s="7"/>
     </row>
     <row r="497">
-      <c r="G497" s="9"/>
+      <c r="C497" s="7"/>
     </row>
     <row r="498">
-      <c r="G498" s="9"/>
+      <c r="C498" s="7"/>
     </row>
     <row r="499">
-      <c r="G499" s="9"/>
+      <c r="C499" s="7"/>
     </row>
     <row r="500">
-      <c r="G500" s="9"/>
+      <c r="C500" s="7"/>
     </row>
     <row r="501">
-      <c r="G501" s="9"/>
+      <c r="C501" s="7"/>
     </row>
     <row r="502">
-      <c r="G502" s="9"/>
+      <c r="C502" s="7"/>
     </row>
     <row r="503">
-      <c r="G503" s="9"/>
+      <c r="C503" s="7"/>
     </row>
     <row r="504">
-      <c r="G504" s="9"/>
+      <c r="C504" s="7"/>
     </row>
     <row r="505">
-      <c r="G505" s="9"/>
+      <c r="C505" s="7"/>
     </row>
     <row r="506">
-      <c r="G506" s="9"/>
+      <c r="C506" s="7"/>
     </row>
     <row r="507">
-      <c r="G507" s="9"/>
+      <c r="C507" s="7"/>
     </row>
     <row r="508">
-      <c r="G508" s="9"/>
+      <c r="C508" s="7"/>
     </row>
     <row r="509">
-      <c r="G509" s="9"/>
+      <c r="C509" s="7"/>
     </row>
     <row r="510">
-      <c r="G510" s="9"/>
+      <c r="C510" s="7"/>
     </row>
     <row r="511">
-      <c r="G511" s="9"/>
+      <c r="C511" s="7"/>
     </row>
     <row r="512">
-      <c r="G512" s="9"/>
+      <c r="C512" s="7"/>
     </row>
     <row r="513">
-      <c r="G513" s="9"/>
+      <c r="C513" s="7"/>
     </row>
     <row r="514">
-      <c r="G514" s="9"/>
+      <c r="C514" s="7"/>
     </row>
     <row r="515">
-      <c r="G515" s="9"/>
+      <c r="C515" s="7"/>
     </row>
     <row r="516">
-      <c r="G516" s="9"/>
+      <c r="C516" s="7"/>
     </row>
     <row r="517">
-      <c r="G517" s="9"/>
+      <c r="C517" s="7"/>
     </row>
     <row r="518">
-      <c r="G518" s="9"/>
+      <c r="C518" s="7"/>
     </row>
     <row r="519">
-      <c r="G519" s="9"/>
+      <c r="C519" s="7"/>
     </row>
     <row r="520">
-      <c r="G520" s="9"/>
+      <c r="C520" s="7"/>
     </row>
     <row r="521">
-      <c r="G521" s="9"/>
+      <c r="C521" s="7"/>
     </row>
     <row r="522">
-      <c r="G522" s="9"/>
+      <c r="C522" s="7"/>
     </row>
     <row r="523">
-      <c r="G523" s="9"/>
+      <c r="C523" s="7"/>
     </row>
     <row r="524">
-      <c r="G524" s="9"/>
+      <c r="C524" s="7"/>
     </row>
     <row r="525">
-      <c r="G525" s="9"/>
+      <c r="C525" s="7"/>
     </row>
     <row r="526">
-      <c r="G526" s="9"/>
+      <c r="C526" s="7"/>
     </row>
     <row r="527">
-      <c r="G527" s="9"/>
+      <c r="C527" s="7"/>
     </row>
     <row r="528">
-      <c r="G528" s="9"/>
+      <c r="C528" s="7"/>
     </row>
     <row r="529">
-      <c r="G529" s="9"/>
+      <c r="C529" s="7"/>
     </row>
     <row r="530">
-      <c r="G530" s="9"/>
+      <c r="C530" s="7"/>
     </row>
     <row r="531">
-      <c r="G531" s="9"/>
+      <c r="C531" s="7"/>
     </row>
     <row r="532">
-      <c r="G532" s="9"/>
+      <c r="C532" s="7"/>
     </row>
     <row r="533">
-      <c r="G533" s="9"/>
+      <c r="C533" s="7"/>
     </row>
     <row r="534">
-      <c r="G534" s="9"/>
+      <c r="C534" s="7"/>
     </row>
     <row r="535">
-      <c r="G535" s="9"/>
+      <c r="C535" s="7"/>
     </row>
     <row r="536">
-      <c r="G536" s="9"/>
+      <c r="C536" s="7"/>
     </row>
     <row r="537">
-      <c r="G537" s="9"/>
+      <c r="C537" s="7"/>
     </row>
     <row r="538">
-      <c r="G538" s="9"/>
+      <c r="C538" s="7"/>
     </row>
     <row r="539">
-      <c r="G539" s="9"/>
+      <c r="C539" s="7"/>
     </row>
     <row r="540">
-      <c r="G540" s="9"/>
+      <c r="C540" s="7"/>
     </row>
     <row r="541">
-      <c r="G541" s="9"/>
+      <c r="C541" s="7"/>
     </row>
     <row r="542">
-      <c r="G542" s="9"/>
+      <c r="C542" s="7"/>
     </row>
     <row r="543">
-      <c r="G543" s="9"/>
+      <c r="C543" s="7"/>
     </row>
     <row r="544">
-      <c r="G544" s="9"/>
+      <c r="C544" s="7"/>
     </row>
     <row r="545">
-      <c r="G545" s="9"/>
+      <c r="C545" s="7"/>
     </row>
     <row r="546">
-      <c r="G546" s="9"/>
+      <c r="C546" s="7"/>
     </row>
     <row r="547">
-      <c r="G547" s="9"/>
+      <c r="C547" s="7"/>
     </row>
     <row r="548">
-      <c r="G548" s="9"/>
+      <c r="C548" s="7"/>
     </row>
     <row r="549">
-      <c r="G549" s="9"/>
+      <c r="C549" s="7"/>
     </row>
     <row r="550">
-      <c r="G550" s="9"/>
+      <c r="C550" s="7"/>
     </row>
     <row r="551">
-      <c r="G551" s="9"/>
+      <c r="C551" s="7"/>
     </row>
     <row r="552">
-      <c r="G552" s="9"/>
+      <c r="C552" s="7"/>
     </row>
     <row r="553">
-      <c r="G553" s="9"/>
+      <c r="C553" s="7"/>
     </row>
     <row r="554">
-      <c r="G554" s="9"/>
+      <c r="C554" s="7"/>
     </row>
     <row r="555">
-      <c r="G555" s="9"/>
+      <c r="C555" s="7"/>
     </row>
     <row r="556">
-      <c r="G556" s="9"/>
+      <c r="C556" s="7"/>
     </row>
     <row r="557">
-      <c r="G557" s="9"/>
+      <c r="C557" s="7"/>
     </row>
     <row r="558">
-      <c r="G558" s="9"/>
+      <c r="C558" s="7"/>
     </row>
     <row r="559">
-      <c r="G559" s="9"/>
+      <c r="C559" s="7"/>
     </row>
     <row r="560">
-      <c r="G560" s="9"/>
+      <c r="C560" s="7"/>
     </row>
     <row r="561">
-      <c r="G561" s="9"/>
+      <c r="C561" s="7"/>
     </row>
     <row r="562">
-      <c r="G562" s="9"/>
+      <c r="C562" s="7"/>
     </row>
     <row r="563">
-      <c r="G563" s="9"/>
+      <c r="C563" s="7"/>
     </row>
     <row r="564">
-      <c r="G564" s="9"/>
+      <c r="C564" s="7"/>
     </row>
     <row r="565">
-      <c r="G565" s="9"/>
+      <c r="C565" s="7"/>
     </row>
     <row r="566">
-      <c r="G566" s="9"/>
+      <c r="C566" s="7"/>
     </row>
     <row r="567">
-      <c r="G567" s="9"/>
+      <c r="C567" s="7"/>
     </row>
     <row r="568">
-      <c r="G568" s="9"/>
+      <c r="C568" s="7"/>
     </row>
     <row r="569">
-      <c r="G569" s="9"/>
+      <c r="C569" s="7"/>
     </row>
     <row r="570">
-      <c r="G570" s="9"/>
+      <c r="C570" s="7"/>
     </row>
     <row r="571">
-      <c r="G571" s="9"/>
+      <c r="C571" s="7"/>
     </row>
     <row r="572">
-      <c r="G572" s="9"/>
+      <c r="C572" s="7"/>
     </row>
     <row r="573">
-      <c r="G573" s="9"/>
+      <c r="C573" s="7"/>
     </row>
     <row r="574">
-      <c r="G574" s="9"/>
+      <c r="C574" s="7"/>
     </row>
     <row r="575">
-      <c r="G575" s="9"/>
+      <c r="C575" s="7"/>
     </row>
     <row r="576">
-      <c r="G576" s="9"/>
+      <c r="C576" s="7"/>
     </row>
     <row r="577">
-      <c r="G577" s="9"/>
+      <c r="C577" s="7"/>
     </row>
     <row r="578">
-      <c r="G578" s="9"/>
+      <c r="C578" s="7"/>
     </row>
     <row r="579">
-      <c r="G579" s="9"/>
+      <c r="C579" s="7"/>
     </row>
     <row r="580">
-      <c r="G580" s="9"/>
+      <c r="C580" s="7"/>
     </row>
     <row r="581">
-      <c r="G581" s="9"/>
+      <c r="C581" s="7"/>
     </row>
     <row r="582">
-      <c r="G582" s="9"/>
+      <c r="C582" s="7"/>
     </row>
     <row r="583">
-      <c r="G583" s="9"/>
+      <c r="C583" s="7"/>
     </row>
     <row r="584">
-      <c r="G584" s="9"/>
+      <c r="C584" s="7"/>
     </row>
     <row r="585">
-      <c r="G585" s="9"/>
+      <c r="C585" s="7"/>
     </row>
     <row r="586">
-      <c r="G586" s="9"/>
+      <c r="C586" s="7"/>
     </row>
     <row r="587">
-      <c r="G587" s="9"/>
+      <c r="C587" s="7"/>
     </row>
     <row r="588">
-      <c r="G588" s="9"/>
+      <c r="C588" s="7"/>
     </row>
     <row r="589">
-      <c r="G589" s="9"/>
+      <c r="C589" s="7"/>
     </row>
     <row r="590">
-      <c r="G590" s="9"/>
+      <c r="C590" s="7"/>
     </row>
     <row r="591">
-      <c r="G591" s="9"/>
+      <c r="C591" s="7"/>
     </row>
     <row r="592">
-      <c r="G592" s="9"/>
+      <c r="C592" s="7"/>
     </row>
     <row r="593">
-      <c r="G593" s="9"/>
+      <c r="C593" s="7"/>
     </row>
     <row r="594">
-      <c r="G594" s="9"/>
+      <c r="C594" s="7"/>
     </row>
     <row r="595">
-      <c r="G595" s="9"/>
+      <c r="C595" s="7"/>
     </row>
     <row r="596">
-      <c r="G596" s="9"/>
+      <c r="C596" s="7"/>
     </row>
     <row r="597">
-      <c r="G597" s="9"/>
+      <c r="C597" s="7"/>
     </row>
     <row r="598">
-      <c r="G598" s="9"/>
+      <c r="C598" s="7"/>
     </row>
     <row r="599">
-      <c r="G599" s="9"/>
+      <c r="C599" s="7"/>
     </row>
     <row r="600">
-      <c r="G600" s="9"/>
+      <c r="C600" s="7"/>
     </row>
     <row r="601">
-      <c r="G601" s="9"/>
+      <c r="C601" s="7"/>
     </row>
     <row r="602">
-      <c r="G602" s="9"/>
+      <c r="C602" s="7"/>
     </row>
     <row r="603">
-      <c r="G603" s="9"/>
+      <c r="C603" s="7"/>
     </row>
     <row r="604">
-      <c r="G604" s="9"/>
+      <c r="C604" s="7"/>
     </row>
     <row r="605">
-      <c r="G605" s="9"/>
+      <c r="C605" s="7"/>
     </row>
     <row r="606">
-      <c r="G606" s="9"/>
+      <c r="C606" s="7"/>
     </row>
     <row r="607">
-      <c r="G607" s="9"/>
+      <c r="C607" s="7"/>
     </row>
     <row r="608">
-      <c r="G608" s="9"/>
+      <c r="C608" s="7"/>
     </row>
     <row r="609">
-      <c r="G609" s="9"/>
+      <c r="C609" s="7"/>
     </row>
     <row r="610">
-      <c r="G610" s="9"/>
+      <c r="C610" s="7"/>
     </row>
     <row r="611">
-      <c r="G611" s="9"/>
+      <c r="C611" s="7"/>
     </row>
     <row r="612">
-      <c r="G612" s="9"/>
+      <c r="C612" s="7"/>
     </row>
     <row r="613">
-      <c r="G613" s="9"/>
+      <c r="C613" s="7"/>
     </row>
     <row r="614">
-      <c r="G614" s="9"/>
+      <c r="C614" s="7"/>
     </row>
     <row r="615">
-      <c r="G615" s="9"/>
+      <c r="C615" s="7"/>
     </row>
     <row r="616">
-      <c r="G616" s="9"/>
+      <c r="C616" s="7"/>
     </row>
     <row r="617">
-      <c r="G617" s="9"/>
+      <c r="C617" s="7"/>
     </row>
     <row r="618">
-      <c r="G618" s="9"/>
+      <c r="C618" s="7"/>
     </row>
     <row r="619">
-      <c r="G619" s="9"/>
+      <c r="C619" s="7"/>
     </row>
     <row r="620">
-      <c r="G620" s="9"/>
+      <c r="C620" s="7"/>
     </row>
     <row r="621">
-      <c r="G621" s="9"/>
+      <c r="C621" s="7"/>
     </row>
     <row r="622">
-      <c r="G622" s="9"/>
+      <c r="C622" s="7"/>
     </row>
     <row r="623">
-      <c r="G623" s="9"/>
+      <c r="C623" s="7"/>
     </row>
     <row r="624">
-      <c r="G624" s="9"/>
+      <c r="C624" s="7"/>
     </row>
     <row r="625">
-      <c r="G625" s="9"/>
+      <c r="C625" s="7"/>
     </row>
     <row r="626">
-      <c r="G626" s="9"/>
+      <c r="C626" s="7"/>
     </row>
     <row r="627">
-      <c r="G627" s="9"/>
+      <c r="C627" s="7"/>
     </row>
     <row r="628">
-      <c r="G628" s="9"/>
+      <c r="C628" s="7"/>
     </row>
     <row r="629">
-      <c r="G629" s="9"/>
+      <c r="C629" s="7"/>
     </row>
     <row r="630">
-      <c r="G630" s="9"/>
+      <c r="C630" s="7"/>
     </row>
     <row r="631">
-      <c r="G631" s="9"/>
+      <c r="C631" s="7"/>
     </row>
     <row r="632">
-      <c r="G632" s="9"/>
+      <c r="C632" s="7"/>
     </row>
     <row r="633">
-      <c r="G633" s="9"/>
+      <c r="C633" s="7"/>
     </row>
     <row r="634">
-      <c r="G634" s="9"/>
+      <c r="C634" s="7"/>
     </row>
     <row r="635">
-      <c r="G635" s="9"/>
+      <c r="C635" s="7"/>
     </row>
     <row r="636">
-      <c r="G636" s="9"/>
+      <c r="C636" s="7"/>
     </row>
     <row r="637">
-      <c r="G637" s="9"/>
+      <c r="C637" s="7"/>
     </row>
     <row r="638">
-      <c r="G638" s="9"/>
+      <c r="C638" s="7"/>
     </row>
     <row r="639">
-      <c r="G639" s="9"/>
+      <c r="C639" s="7"/>
     </row>
     <row r="640">
-      <c r="G640" s="9"/>
+      <c r="C640" s="7"/>
     </row>
     <row r="641">
-      <c r="G641" s="9"/>
+      <c r="C641" s="7"/>
     </row>
     <row r="642">
-      <c r="G642" s="9"/>
+      <c r="C642" s="7"/>
     </row>
     <row r="643">
-      <c r="G643" s="9"/>
+      <c r="C643" s="7"/>
     </row>
     <row r="644">
-      <c r="G644" s="9"/>
+      <c r="C644" s="7"/>
     </row>
     <row r="645">
-      <c r="G645" s="9"/>
+      <c r="C645" s="7"/>
     </row>
     <row r="646">
-      <c r="G646" s="9"/>
+      <c r="C646" s="7"/>
     </row>
     <row r="647">
-      <c r="G647" s="9"/>
+      <c r="C647" s="7"/>
     </row>
     <row r="648">
-      <c r="G648" s="9"/>
+      <c r="C648" s="7"/>
     </row>
     <row r="649">
-      <c r="G649" s="9"/>
+      <c r="C649" s="7"/>
     </row>
     <row r="650">
-      <c r="G650" s="9"/>
+      <c r="C650" s="7"/>
     </row>
     <row r="651">
-      <c r="G651" s="9"/>
+      <c r="C651" s="7"/>
     </row>
     <row r="652">
-      <c r="G652" s="9"/>
+      <c r="C652" s="7"/>
     </row>
     <row r="653">
-      <c r="G653" s="9"/>
+      <c r="C653" s="7"/>
     </row>
     <row r="654">
-      <c r="G654" s="9"/>
+      <c r="C654" s="7"/>
     </row>
     <row r="655">
-      <c r="G655" s="9"/>
+      <c r="C655" s="7"/>
     </row>
     <row r="656">
-      <c r="G656" s="9"/>
+      <c r="C656" s="7"/>
     </row>
     <row r="657">
-      <c r="G657" s="9"/>
+      <c r="C657" s="7"/>
     </row>
     <row r="658">
-      <c r="G658" s="9"/>
+      <c r="C658" s="7"/>
     </row>
     <row r="659">
-      <c r="G659" s="9"/>
+      <c r="C659" s="7"/>
     </row>
     <row r="660">
-      <c r="G660" s="9"/>
+      <c r="C660" s="7"/>
     </row>
     <row r="661">
-      <c r="G661" s="9"/>
+      <c r="C661" s="7"/>
     </row>
     <row r="662">
-      <c r="G662" s="9"/>
+      <c r="C662" s="7"/>
     </row>
     <row r="663">
-      <c r="G663" s="9"/>
+      <c r="C663" s="7"/>
     </row>
     <row r="664">
-      <c r="G664" s="9"/>
+      <c r="C664" s="7"/>
     </row>
     <row r="665">
-      <c r="G665" s="9"/>
+      <c r="C665" s="7"/>
     </row>
     <row r="666">
-      <c r="G666" s="9"/>
+      <c r="C666" s="7"/>
     </row>
     <row r="667">
-      <c r="G667" s="9"/>
+      <c r="C667" s="7"/>
     </row>
     <row r="668">
-      <c r="G668" s="9"/>
+      <c r="C668" s="7"/>
     </row>
     <row r="669">
-      <c r="G669" s="9"/>
+      <c r="C669" s="7"/>
     </row>
     <row r="670">
-      <c r="G670" s="9"/>
+      <c r="C670" s="7"/>
     </row>
     <row r="671">
-      <c r="G671" s="9"/>
+      <c r="C671" s="7"/>
     </row>
     <row r="672">
-      <c r="G672" s="9"/>
+      <c r="C672" s="7"/>
     </row>
     <row r="673">
-      <c r="G673" s="9"/>
+      <c r="C673" s="7"/>
     </row>
     <row r="674">
-      <c r="G674" s="9"/>
+      <c r="C674" s="7"/>
     </row>
     <row r="675">
-      <c r="G675" s="9"/>
+      <c r="C675" s="7"/>
     </row>
     <row r="676">
-      <c r="G676" s="9"/>
+      <c r="C676" s="7"/>
     </row>
     <row r="677">
-      <c r="G677" s="9"/>
+      <c r="C677" s="7"/>
     </row>
     <row r="678">
-      <c r="G678" s="9"/>
+      <c r="C678" s="7"/>
     </row>
     <row r="679">
-      <c r="G679" s="9"/>
+      <c r="C679" s="7"/>
     </row>
     <row r="680">
-      <c r="G680" s="9"/>
+      <c r="C680" s="7"/>
     </row>
     <row r="681">
-      <c r="G681" s="9"/>
+      <c r="C681" s="7"/>
     </row>
     <row r="682">
-      <c r="G682" s="9"/>
+      <c r="C682" s="7"/>
     </row>
     <row r="683">
-      <c r="G683" s="9"/>
+      <c r="C683" s="7"/>
     </row>
     <row r="684">
-      <c r="G684" s="9"/>
+      <c r="C684" s="7"/>
     </row>
     <row r="685">
-      <c r="G685" s="9"/>
+      <c r="C685" s="7"/>
     </row>
     <row r="686">
-      <c r="G686" s="9"/>
+      <c r="C686" s="7"/>
     </row>
     <row r="687">
-      <c r="G687" s="9"/>
+      <c r="C687" s="7"/>
     </row>
     <row r="688">
-      <c r="G688" s="9"/>
+      <c r="C688" s="7"/>
     </row>
     <row r="689">
-      <c r="G689" s="9"/>
+      <c r="C689" s="7"/>
     </row>
     <row r="690">
-      <c r="G690" s="9"/>
+      <c r="C690" s="7"/>
     </row>
     <row r="691">
-      <c r="G691" s="9"/>
+      <c r="C691" s="7"/>
     </row>
     <row r="692">
-      <c r="G692" s="9"/>
+      <c r="C692" s="7"/>
     </row>
     <row r="693">
-      <c r="G693" s="9"/>
+      <c r="C693" s="7"/>
     </row>
     <row r="694">
-      <c r="G694" s="9"/>
+      <c r="C694" s="7"/>
     </row>
     <row r="695">
-      <c r="G695" s="9"/>
+      <c r="C695" s="7"/>
     </row>
     <row r="696">
-      <c r="G696" s="9"/>
+      <c r="C696" s="7"/>
     </row>
     <row r="697">
-      <c r="G697" s="9"/>
+      <c r="C697" s="7"/>
     </row>
     <row r="698">
-      <c r="G698" s="9"/>
+      <c r="C698" s="7"/>
     </row>
     <row r="699">
-      <c r="G699" s="9"/>
+      <c r="C699" s="7"/>
     </row>
     <row r="700">
-      <c r="G700" s="9"/>
+      <c r="C700" s="7"/>
     </row>
     <row r="701">
-      <c r="G701" s="9"/>
+      <c r="C701" s="7"/>
     </row>
     <row r="702">
-      <c r="G702" s="9"/>
+      <c r="C702" s="7"/>
     </row>
     <row r="703">
-      <c r="G703" s="9"/>
+      <c r="C703" s="7"/>
     </row>
     <row r="704">
-      <c r="G704" s="9"/>
+      <c r="C704" s="7"/>
     </row>
     <row r="705">
-      <c r="G705" s="9"/>
+      <c r="C705" s="7"/>
     </row>
     <row r="706">
-      <c r="G706" s="9"/>
+      <c r="C706" s="7"/>
     </row>
     <row r="707">
-      <c r="G707" s="9"/>
+      <c r="C707" s="7"/>
     </row>
     <row r="708">
-      <c r="G708" s="9"/>
+      <c r="C708" s="7"/>
     </row>
     <row r="709">
-      <c r="G709" s="9"/>
+      <c r="C709" s="7"/>
     </row>
     <row r="710">
-      <c r="G710" s="9"/>
+      <c r="C710" s="7"/>
     </row>
     <row r="711">
-      <c r="G711" s="9"/>
+      <c r="C711" s="7"/>
     </row>
     <row r="712">
-      <c r="G712" s="9"/>
+      <c r="C712" s="7"/>
     </row>
     <row r="713">
-      <c r="G713" s="9"/>
+      <c r="C713" s="7"/>
     </row>
     <row r="714">
-      <c r="G714" s="9"/>
+      <c r="C714" s="7"/>
     </row>
     <row r="715">
-      <c r="G715" s="9"/>
+      <c r="C715" s="7"/>
     </row>
     <row r="716">
-      <c r="G716" s="9"/>
+      <c r="C716" s="7"/>
     </row>
     <row r="717">
-      <c r="G717" s="9"/>
+      <c r="C717" s="7"/>
     </row>
     <row r="718">
-      <c r="G718" s="9"/>
+      <c r="C718" s="7"/>
     </row>
     <row r="719">
-      <c r="G719" s="9"/>
+      <c r="C719" s="7"/>
     </row>
     <row r="720">
-      <c r="G720" s="9"/>
+      <c r="C720" s="7"/>
     </row>
     <row r="721">
-      <c r="G721" s="9"/>
+      <c r="C721" s="7"/>
     </row>
     <row r="722">
-      <c r="G722" s="9"/>
+      <c r="C722" s="7"/>
     </row>
     <row r="723">
-      <c r="G723" s="9"/>
+      <c r="C723" s="7"/>
     </row>
     <row r="724">
-      <c r="G724" s="9"/>
+      <c r="C724" s="7"/>
     </row>
     <row r="725">
-      <c r="G725" s="9"/>
+      <c r="C725" s="7"/>
     </row>
     <row r="726">
-      <c r="G726" s="9"/>
+      <c r="C726" s="7"/>
     </row>
     <row r="727">
-      <c r="G727" s="9"/>
+      <c r="C727" s="7"/>
     </row>
     <row r="728">
-      <c r="G728" s="9"/>
+      <c r="C728" s="7"/>
     </row>
     <row r="729">
-      <c r="G729" s="9"/>
+      <c r="C729" s="7"/>
     </row>
     <row r="730">
-      <c r="G730" s="9"/>
+      <c r="C730" s="7"/>
     </row>
     <row r="731">
-      <c r="G731" s="9"/>
+      <c r="C731" s="7"/>
     </row>
     <row r="732">
-      <c r="G732" s="9"/>
+      <c r="C732" s="7"/>
     </row>
     <row r="733">
-      <c r="G733" s="9"/>
+      <c r="C733" s="7"/>
     </row>
     <row r="734">
-      <c r="G734" s="9"/>
+      <c r="C734" s="7"/>
     </row>
     <row r="735">
-      <c r="G735" s="9"/>
+      <c r="C735" s="7"/>
     </row>
     <row r="736">
-      <c r="G736" s="9"/>
+      <c r="C736" s="7"/>
     </row>
     <row r="737">
-      <c r="G737" s="9"/>
+      <c r="C737" s="7"/>
     </row>
     <row r="738">
-      <c r="G738" s="9"/>
+      <c r="C738" s="7"/>
     </row>
     <row r="739">
-      <c r="G739" s="9"/>
+      <c r="C739" s="7"/>
     </row>
     <row r="740">
-      <c r="G740" s="9"/>
+      <c r="C740" s="7"/>
     </row>
     <row r="741">
-      <c r="G741" s="9"/>
+      <c r="C741" s="7"/>
     </row>
     <row r="742">
-      <c r="G742" s="9"/>
+      <c r="C742" s="7"/>
     </row>
     <row r="743">
-      <c r="G743" s="9"/>
+      <c r="C743" s="7"/>
     </row>
     <row r="744">
-      <c r="G744" s="9"/>
+      <c r="C744" s="7"/>
     </row>
     <row r="745">
-      <c r="G745" s="9"/>
+      <c r="C745" s="7"/>
     </row>
     <row r="746">
-      <c r="G746" s="9"/>
+      <c r="C746" s="7"/>
     </row>
     <row r="747">
-      <c r="G747" s="9"/>
+      <c r="C747" s="7"/>
     </row>
     <row r="748">
-      <c r="G748" s="9"/>
+      <c r="C748" s="7"/>
     </row>
     <row r="749">
-      <c r="G749" s="9"/>
+      <c r="C749" s="7"/>
     </row>
     <row r="750">
-      <c r="G750" s="9"/>
+      <c r="C750" s="7"/>
     </row>
     <row r="751">
-      <c r="G751" s="9"/>
+      <c r="C751" s="7"/>
     </row>
     <row r="752">
-      <c r="G752" s="9"/>
+      <c r="C752" s="7"/>
     </row>
     <row r="753">
-      <c r="G753" s="9"/>
+      <c r="C753" s="7"/>
     </row>
     <row r="754">
-      <c r="G754" s="9"/>
+      <c r="C754" s="7"/>
     </row>
     <row r="755">
-      <c r="G755" s="9"/>
+      <c r="C755" s="7"/>
     </row>
     <row r="756">
-      <c r="G756" s="9"/>
+      <c r="C756" s="7"/>
     </row>
     <row r="757">
-      <c r="G757" s="9"/>
+      <c r="C757" s="7"/>
     </row>
     <row r="758">
-      <c r="G758" s="9"/>
+      <c r="C758" s="7"/>
     </row>
     <row r="759">
-      <c r="G759" s="9"/>
+      <c r="C759" s="7"/>
     </row>
     <row r="760">
-      <c r="G760" s="9"/>
+      <c r="C760" s="7"/>
     </row>
     <row r="761">
-      <c r="G761" s="9"/>
+      <c r="C761" s="7"/>
     </row>
     <row r="762">
-      <c r="G762" s="9"/>
+      <c r="C762" s="7"/>
     </row>
     <row r="763">
-      <c r="G763" s="9"/>
+      <c r="C763" s="7"/>
     </row>
     <row r="764">
-      <c r="G764" s="9"/>
+      <c r="C764" s="7"/>
     </row>
     <row r="765">
-      <c r="G765" s="9"/>
+      <c r="C765" s="7"/>
     </row>
     <row r="766">
-      <c r="G766" s="9"/>
+      <c r="C766" s="7"/>
     </row>
     <row r="767">
-      <c r="G767" s="9"/>
+      <c r="C767" s="7"/>
     </row>
     <row r="768">
-      <c r="G768" s="9"/>
+      <c r="C768" s="7"/>
     </row>
     <row r="769">
-      <c r="G769" s="9"/>
+      <c r="C769" s="7"/>
     </row>
     <row r="770">
-      <c r="G770" s="9"/>
+      <c r="C770" s="7"/>
     </row>
     <row r="771">
-      <c r="G771" s="9"/>
+      <c r="C771" s="7"/>
     </row>
     <row r="772">
-      <c r="G772" s="9"/>
+      <c r="C772" s="7"/>
     </row>
     <row r="773">
-      <c r="G773" s="9"/>
+      <c r="C773" s="7"/>
     </row>
     <row r="774">
-      <c r="G774" s="9"/>
+      <c r="C774" s="7"/>
     </row>
     <row r="775">
-      <c r="G775" s="9"/>
+      <c r="C775" s="7"/>
     </row>
     <row r="776">
-      <c r="G776" s="9"/>
+      <c r="C776" s="7"/>
     </row>
     <row r="777">
-      <c r="G777" s="9"/>
+      <c r="C777" s="7"/>
     </row>
     <row r="778">
-      <c r="G778" s="9"/>
+      <c r="C778" s="7"/>
     </row>
     <row r="779">
-      <c r="G779" s="9"/>
+      <c r="C779" s="7"/>
     </row>
     <row r="780">
-      <c r="G780" s="9"/>
+      <c r="C780" s="7"/>
     </row>
     <row r="781">
-      <c r="G781" s="9"/>
+      <c r="C781" s="7"/>
     </row>
     <row r="782">
-      <c r="G782" s="9"/>
+      <c r="C782" s="7"/>
     </row>
     <row r="783">
-      <c r="G783" s="9"/>
+      <c r="C783" s="7"/>
     </row>
     <row r="784">
-      <c r="G784" s="9"/>
+      <c r="C784" s="7"/>
     </row>
     <row r="785">
-      <c r="G785" s="9"/>
+      <c r="C785" s="7"/>
     </row>
     <row r="786">
-      <c r="G786" s="9"/>
+      <c r="C786" s="7"/>
     </row>
     <row r="787">
-      <c r="G787" s="9"/>
+      <c r="C787" s="7"/>
     </row>
     <row r="788">
-      <c r="G788" s="9"/>
+      <c r="C788" s="7"/>
     </row>
     <row r="789">
-      <c r="G789" s="9"/>
+      <c r="C789" s="7"/>
     </row>
     <row r="790">
-      <c r="G790" s="9"/>
+      <c r="C790" s="7"/>
     </row>
     <row r="791">
-      <c r="G791" s="9"/>
+      <c r="C791" s="7"/>
     </row>
     <row r="792">
-      <c r="G792" s="9"/>
+      <c r="C792" s="7"/>
     </row>
     <row r="793">
-      <c r="G793" s="9"/>
+      <c r="C793" s="7"/>
     </row>
     <row r="794">
-      <c r="G794" s="9"/>
+      <c r="C794" s="7"/>
     </row>
     <row r="795">
-      <c r="G795" s="9"/>
+      <c r="C795" s="7"/>
     </row>
     <row r="796">
-      <c r="G796" s="9"/>
+      <c r="C796" s="7"/>
     </row>
     <row r="797">
-      <c r="G797" s="9"/>
+      <c r="C797" s="7"/>
     </row>
     <row r="798">
-      <c r="G798" s="9"/>
+      <c r="C798" s="7"/>
     </row>
     <row r="799">
-      <c r="G799" s="9"/>
+      <c r="C799" s="7"/>
     </row>
     <row r="800">
-      <c r="G800" s="9"/>
+      <c r="C800" s="7"/>
     </row>
     <row r="801">
-      <c r="G801" s="9"/>
+      <c r="C801" s="7"/>
     </row>
     <row r="802">
-      <c r="G802" s="9"/>
+      <c r="C802" s="7"/>
     </row>
     <row r="803">
-      <c r="G803" s="9"/>
+      <c r="C803" s="7"/>
     </row>
     <row r="804">
-      <c r="G804" s="9"/>
+      <c r="C804" s="7"/>
     </row>
     <row r="805">
-      <c r="G805" s="9"/>
+      <c r="C805" s="7"/>
     </row>
     <row r="806">
-      <c r="G806" s="9"/>
+      <c r="C806" s="7"/>
     </row>
     <row r="807">
-      <c r="G807" s="9"/>
+      <c r="C807" s="7"/>
     </row>
     <row r="808">
-      <c r="G808" s="9"/>
+      <c r="C808" s="7"/>
     </row>
     <row r="809">
-      <c r="G809" s="9"/>
+      <c r="C809" s="7"/>
     </row>
     <row r="810">
-      <c r="G810" s="9"/>
+      <c r="C810" s="7"/>
     </row>
     <row r="811">
-      <c r="G811" s="9"/>
+      <c r="C811" s="7"/>
     </row>
     <row r="812">
-      <c r="G812" s="9"/>
+      <c r="C812" s="7"/>
     </row>
     <row r="813">
-      <c r="G813" s="9"/>
+      <c r="C813" s="7"/>
     </row>
     <row r="814">
-      <c r="G814" s="9"/>
+      <c r="C814" s="7"/>
     </row>
     <row r="815">
-      <c r="G815" s="9"/>
+      <c r="C815" s="7"/>
     </row>
     <row r="816">
-      <c r="G816" s="9"/>
+      <c r="C816" s="7"/>
     </row>
     <row r="817">
-      <c r="G817" s="9"/>
+      <c r="C817" s="7"/>
     </row>
     <row r="818">
-      <c r="G818" s="9"/>
+      <c r="C818" s="7"/>
     </row>
     <row r="819">
-      <c r="G819" s="9"/>
+      <c r="C819" s="7"/>
     </row>
     <row r="820">
-      <c r="G820" s="9"/>
+      <c r="C820" s="7"/>
     </row>
     <row r="821">
-      <c r="G821" s="9"/>
+      <c r="C821" s="7"/>
     </row>
     <row r="822">
-      <c r="G822" s="9"/>
+      <c r="C822" s="7"/>
     </row>
     <row r="823">
-      <c r="G823" s="9"/>
+      <c r="C823" s="7"/>
     </row>
     <row r="824">
-      <c r="G824" s="9"/>
+      <c r="C824" s="7"/>
     </row>
     <row r="825">
-      <c r="G825" s="9"/>
+      <c r="C825" s="7"/>
     </row>
     <row r="826">
-      <c r="G826" s="9"/>
+      <c r="C826" s="7"/>
     </row>
     <row r="827">
-      <c r="G827" s="9"/>
+      <c r="C827" s="7"/>
     </row>
     <row r="828">
-      <c r="G828" s="9"/>
+      <c r="C828" s="7"/>
     </row>
     <row r="829">
-      <c r="G829" s="9"/>
+      <c r="C829" s="7"/>
     </row>
     <row r="830">
-      <c r="G830" s="9"/>
+      <c r="C830" s="7"/>
     </row>
     <row r="831">
-      <c r="G831" s="9"/>
+      <c r="C831" s="7"/>
     </row>
     <row r="832">
-      <c r="G832" s="9"/>
+      <c r="C832" s="7"/>
     </row>
     <row r="833">
-      <c r="G833" s="9"/>
+      <c r="C833" s="7"/>
     </row>
     <row r="834">
-      <c r="G834" s="9"/>
+      <c r="C834" s="7"/>
     </row>
     <row r="835">
-      <c r="G835" s="9"/>
+      <c r="C835" s="7"/>
     </row>
     <row r="836">
-      <c r="G836" s="9"/>
+      <c r="C836" s="7"/>
     </row>
     <row r="837">
-      <c r="G837" s="9"/>
+      <c r="C837" s="7"/>
     </row>
     <row r="838">
-      <c r="G838" s="9"/>
+      <c r="C838" s="7"/>
     </row>
     <row r="839">
-      <c r="G839" s="9"/>
+      <c r="C839" s="7"/>
     </row>
     <row r="840">
-      <c r="G840" s="9"/>
+      <c r="C840" s="7"/>
     </row>
     <row r="841">
-      <c r="G841" s="9"/>
+      <c r="C841" s="7"/>
     </row>
     <row r="842">
-      <c r="G842" s="9"/>
+      <c r="C842" s="7"/>
     </row>
     <row r="843">
-      <c r="G843" s="9"/>
+      <c r="C843" s="7"/>
     </row>
     <row r="844">
-      <c r="G844" s="9"/>
+      <c r="C844" s="7"/>
     </row>
     <row r="845">
-      <c r="G845" s="9"/>
+      <c r="C845" s="7"/>
     </row>
     <row r="846">
-      <c r="G846" s="9"/>
+      <c r="C846" s="7"/>
     </row>
     <row r="847">
-      <c r="G847" s="9"/>
+      <c r="C847" s="7"/>
     </row>
     <row r="848">
-      <c r="G848" s="9"/>
+      <c r="C848" s="7"/>
     </row>
     <row r="849">
-      <c r="G849" s="9"/>
+      <c r="C849" s="7"/>
     </row>
     <row r="850">
-      <c r="G850" s="9"/>
+      <c r="C850" s="7"/>
     </row>
     <row r="851">
-      <c r="G851" s="9"/>
+      <c r="C851" s="7"/>
     </row>
     <row r="852">
-      <c r="G852" s="9"/>
+      <c r="C852" s="7"/>
     </row>
     <row r="853">
-      <c r="G853" s="9"/>
+      <c r="C853" s="7"/>
     </row>
     <row r="854">
-      <c r="G854" s="9"/>
+      <c r="C854" s="7"/>
     </row>
     <row r="855">
-      <c r="G855" s="9"/>
+      <c r="C855" s="7"/>
     </row>
     <row r="856">
-      <c r="G856" s="9"/>
+      <c r="C856" s="7"/>
     </row>
     <row r="857">
-      <c r="G857" s="9"/>
+      <c r="C857" s="7"/>
     </row>
     <row r="858">
-      <c r="G858" s="9"/>
+      <c r="C858" s="7"/>
     </row>
     <row r="859">
-      <c r="G859" s="9"/>
+      <c r="C859" s="7"/>
     </row>
     <row r="860">
-      <c r="G860" s="9"/>
+      <c r="C860" s="7"/>
     </row>
     <row r="861">
-      <c r="G861" s="9"/>
+      <c r="C861" s="7"/>
     </row>
     <row r="862">
-      <c r="G862" s="9"/>
+      <c r="C862" s="7"/>
     </row>
     <row r="863">
-      <c r="G863" s="9"/>
+      <c r="C863" s="7"/>
     </row>
     <row r="864">
-      <c r="G864" s="9"/>
+      <c r="C864" s="7"/>
     </row>
     <row r="865">
-      <c r="G865" s="9"/>
+      <c r="C865" s="7"/>
     </row>
     <row r="866">
-      <c r="G866" s="9"/>
+      <c r="C866" s="7"/>
     </row>
     <row r="867">
-      <c r="G867" s="9"/>
+      <c r="C867" s="7"/>
     </row>
     <row r="868">
-      <c r="G868" s="9"/>
+      <c r="C868" s="7"/>
     </row>
     <row r="869">
-      <c r="G869" s="9"/>
+      <c r="C869" s="7"/>
     </row>
     <row r="870">
-      <c r="G870" s="9"/>
+      <c r="C870" s="7"/>
     </row>
     <row r="871">
-      <c r="G871" s="9"/>
+      <c r="C871" s="7"/>
     </row>
     <row r="872">
-      <c r="G872" s="9"/>
+      <c r="C872" s="7"/>
     </row>
     <row r="873">
-      <c r="G873" s="9"/>
+      <c r="C873" s="7"/>
     </row>
     <row r="874">
-      <c r="G874" s="9"/>
+      <c r="C874" s="7"/>
     </row>
     <row r="875">
-      <c r="G875" s="9"/>
+      <c r="C875" s="7"/>
     </row>
     <row r="876">
-      <c r="G876" s="9"/>
+      <c r="C876" s="7"/>
     </row>
     <row r="877">
-      <c r="G877" s="9"/>
+      <c r="C877" s="7"/>
     </row>
     <row r="878">
-      <c r="G878" s="9"/>
+      <c r="C878" s="7"/>
     </row>
     <row r="879">
-      <c r="G879" s="9"/>
+      <c r="C879" s="7"/>
     </row>
     <row r="880">
-      <c r="G880" s="9"/>
+      <c r="C880" s="7"/>
     </row>
     <row r="881">
-      <c r="G881" s="9"/>
+      <c r="C881" s="7"/>
     </row>
     <row r="882">
-      <c r="G882" s="9"/>
+      <c r="C882" s="7"/>
     </row>
     <row r="883">
-      <c r="G883" s="9"/>
+      <c r="C883" s="7"/>
     </row>
     <row r="884">
-      <c r="G884" s="9"/>
+      <c r="C884" s="7"/>
     </row>
     <row r="885">
-      <c r="G885" s="9"/>
+      <c r="C885" s="7"/>
     </row>
     <row r="886">
-      <c r="G886" s="9"/>
+      <c r="C886" s="7"/>
     </row>
     <row r="887">
-      <c r="G887" s="9"/>
+      <c r="C887" s="7"/>
     </row>
     <row r="888">
-      <c r="G888" s="9"/>
+      <c r="C888" s="7"/>
     </row>
     <row r="889">
-      <c r="G889" s="9"/>
+      <c r="C889" s="7"/>
     </row>
     <row r="890">
-      <c r="G890" s="9"/>
+      <c r="C890" s="7"/>
     </row>
     <row r="891">
-      <c r="G891" s="9"/>
+      <c r="C891" s="7"/>
     </row>
     <row r="892">
-      <c r="G892" s="9"/>
+      <c r="C892" s="7"/>
     </row>
     <row r="893">
-      <c r="G893" s="9"/>
+      <c r="C893" s="7"/>
     </row>
     <row r="894">
-      <c r="G894" s="9"/>
+      <c r="C894" s="7"/>
     </row>
     <row r="895">
-      <c r="G895" s="9"/>
+      <c r="C895" s="7"/>
     </row>
     <row r="896">
-      <c r="G896" s="9"/>
+      <c r="C896" s="7"/>
     </row>
     <row r="897">
-      <c r="G897" s="9"/>
+      <c r="C897" s="7"/>
     </row>
     <row r="898">
-      <c r="G898" s="9"/>
+      <c r="C898" s="7"/>
     </row>
     <row r="899">
-      <c r="G899" s="9"/>
+      <c r="C899" s="7"/>
     </row>
     <row r="900">
-      <c r="G900" s="9"/>
+      <c r="C900" s="7"/>
     </row>
     <row r="901">
-      <c r="G901" s="9"/>
+      <c r="C901" s="7"/>
     </row>
     <row r="902">
-      <c r="G902" s="9"/>
+      <c r="C902" s="7"/>
     </row>
     <row r="903">
-      <c r="G903" s="9"/>
+      <c r="C903" s="7"/>
     </row>
     <row r="904">
-      <c r="G904" s="9"/>
+      <c r="C904" s="7"/>
     </row>
     <row r="905">
-      <c r="G905" s="9"/>
+      <c r="C905" s="7"/>
     </row>
     <row r="906">
-      <c r="G906" s="9"/>
+      <c r="C906" s="7"/>
     </row>
     <row r="907">
-      <c r="G907" s="9"/>
+      <c r="C907" s="7"/>
     </row>
     <row r="908">
-      <c r="G908" s="9"/>
+      <c r="C908" s="7"/>
     </row>
     <row r="909">
-      <c r="G909" s="9"/>
+      <c r="C909" s="7"/>
     </row>
     <row r="910">
-      <c r="G910" s="9"/>
+      <c r="C910" s="7"/>
     </row>
     <row r="911">
-      <c r="G911" s="9"/>
+      <c r="C911" s="7"/>
     </row>
     <row r="912">
-      <c r="G912" s="9"/>
+      <c r="C912" s="7"/>
     </row>
     <row r="913">
-      <c r="G913" s="9"/>
+      <c r="C913" s="7"/>
     </row>
     <row r="914">
-      <c r="G914" s="9"/>
+      <c r="C914" s="7"/>
     </row>
     <row r="915">
-      <c r="G915" s="9"/>
+      <c r="C915" s="7"/>
     </row>
     <row r="916">
-      <c r="G916" s="9"/>
+      <c r="C916" s="7"/>
     </row>
     <row r="917">
-      <c r="G917" s="9"/>
+      <c r="C917" s="7"/>
     </row>
     <row r="918">
-      <c r="G918" s="9"/>
+      <c r="C918" s="7"/>
     </row>
     <row r="919">
-      <c r="G919" s="9"/>
+      <c r="C919" s="7"/>
     </row>
     <row r="920">
-      <c r="G920" s="9"/>
+      <c r="C920" s="7"/>
     </row>
     <row r="921">
-      <c r="G921" s="9"/>
+      <c r="C921" s="7"/>
     </row>
     <row r="922">
-      <c r="G922" s="9"/>
+      <c r="C922" s="7"/>
     </row>
     <row r="923">
-      <c r="G923" s="9"/>
+      <c r="C923" s="7"/>
     </row>
     <row r="924">
-      <c r="G924" s="9"/>
+      <c r="C924" s="7"/>
     </row>
     <row r="925">
-      <c r="G925" s="9"/>
+      <c r="C925" s="7"/>
     </row>
     <row r="926">
-      <c r="G926" s="9"/>
+      <c r="C926" s="7"/>
     </row>
     <row r="927">
-      <c r="G927" s="9"/>
+      <c r="C927" s="7"/>
     </row>
     <row r="928">
-      <c r="G928" s="9"/>
+      <c r="C928" s="7"/>
     </row>
     <row r="929">
-      <c r="G929" s="9"/>
+      <c r="C929" s="7"/>
     </row>
     <row r="930">
-      <c r="G930" s="9"/>
+      <c r="C930" s="7"/>
     </row>
     <row r="931">
-      <c r="G931" s="9"/>
+      <c r="C931" s="7"/>
     </row>
     <row r="932">
-      <c r="G932" s="9"/>
+      <c r="C932" s="7"/>
     </row>
     <row r="933">
-      <c r="G933" s="9"/>
+      <c r="C933" s="7"/>
     </row>
     <row r="934">
-      <c r="G934" s="9"/>
+      <c r="C934" s="7"/>
     </row>
     <row r="935">
-      <c r="G935" s="9"/>
+      <c r="C935" s="7"/>
     </row>
     <row r="936">
-      <c r="G936" s="9"/>
+      <c r="C936" s="7"/>
     </row>
     <row r="937">
-      <c r="G937" s="9"/>
+      <c r="C937" s="7"/>
     </row>
     <row r="938">
-      <c r="G938" s="9"/>
+      <c r="C938" s="7"/>
     </row>
     <row r="939">
-      <c r="G939" s="9"/>
+      <c r="C939" s="7"/>
     </row>
     <row r="940">
-      <c r="G940" s="9"/>
+      <c r="C940" s="7"/>
     </row>
     <row r="941">
-      <c r="G941" s="9"/>
+      <c r="C941" s="7"/>
     </row>
     <row r="942">
-      <c r="G942" s="9"/>
+      <c r="C942" s="7"/>
     </row>
     <row r="943">
-      <c r="G943" s="9"/>
+      <c r="C943" s="7"/>
     </row>
     <row r="944">
-      <c r="G944" s="9"/>
+      <c r="C944" s="7"/>
     </row>
     <row r="945">
-      <c r="G945" s="9"/>
+      <c r="C945" s="7"/>
     </row>
     <row r="946">
-      <c r="G946" s="9"/>
+      <c r="C946" s="7"/>
     </row>
     <row r="947">
-      <c r="G947" s="9"/>
+      <c r="C947" s="7"/>
     </row>
     <row r="948">
-      <c r="G948" s="9"/>
+      <c r="C948" s="7"/>
     </row>
     <row r="949">
-      <c r="G949" s="9"/>
+      <c r="C949" s="7"/>
     </row>
     <row r="950">
-      <c r="G950" s="9"/>
+      <c r="C950" s="7"/>
     </row>
     <row r="951">
-      <c r="G951" s="9"/>
+      <c r="C951" s="7"/>
     </row>
     <row r="952">
-      <c r="G952" s="9"/>
+      <c r="C952" s="7"/>
     </row>
     <row r="953">
-      <c r="G953" s="9"/>
+      <c r="C953" s="7"/>
     </row>
     <row r="954">
-      <c r="G954" s="9"/>
+      <c r="C954" s="7"/>
     </row>
     <row r="955">
-      <c r="G955" s="9"/>
+      <c r="C955" s="7"/>
     </row>
     <row r="956">
-      <c r="G956" s="9"/>
+      <c r="C956" s="7"/>
     </row>
     <row r="957">
-      <c r="G957" s="9"/>
+      <c r="C957" s="7"/>
     </row>
     <row r="958">
-      <c r="G958" s="9"/>
+      <c r="C958" s="7"/>
     </row>
     <row r="959">
-      <c r="G959" s="9"/>
+      <c r="C959" s="7"/>
     </row>
     <row r="960">
-      <c r="G960" s="9"/>
+      <c r="C960" s="7"/>
     </row>
     <row r="961">
-      <c r="G961" s="9"/>
+      <c r="C961" s="7"/>
     </row>
     <row r="962">
-      <c r="G962" s="9"/>
+      <c r="C962" s="7"/>
     </row>
     <row r="963">
-      <c r="G963" s="9"/>
+      <c r="C963" s="7"/>
     </row>
     <row r="964">
-      <c r="G964" s="9"/>
+      <c r="C964" s="7"/>
     </row>
     <row r="965">
-      <c r="G965" s="9"/>
+      <c r="C965" s="7"/>
     </row>
     <row r="966">
-      <c r="G966" s="9"/>
+      <c r="C966" s="7"/>
     </row>
     <row r="967">
-      <c r="G967" s="9"/>
+      <c r="C967" s="7"/>
     </row>
     <row r="968">
-      <c r="G968" s="9"/>
+      <c r="C968" s="7"/>
     </row>
     <row r="969">
-      <c r="G969" s="9"/>
+      <c r="C969" s="7"/>
     </row>
     <row r="970">
-      <c r="G970" s="9"/>
+      <c r="C970" s="7"/>
     </row>
     <row r="971">
-      <c r="G971" s="9"/>
+      <c r="C971" s="7"/>
     </row>
     <row r="972">
-      <c r="G972" s="9"/>
+      <c r="C972" s="7"/>
     </row>
     <row r="973">
-      <c r="G973" s="9"/>
+      <c r="C973" s="7"/>
     </row>
     <row r="974">
-      <c r="G974" s="9"/>
+      <c r="C974" s="7"/>
     </row>
     <row r="975">
-      <c r="G975" s="9"/>
+      <c r="C975" s="7"/>
     </row>
     <row r="976">
-      <c r="G976" s="9"/>
+      <c r="C976" s="7"/>
     </row>
     <row r="977">
-      <c r="G977" s="9"/>
+      <c r="C977" s="7"/>
     </row>
     <row r="978">
-      <c r="G978" s="9"/>
+      <c r="C978" s="7"/>
     </row>
     <row r="979">
-      <c r="G979" s="9"/>
+      <c r="C979" s="7"/>
     </row>
     <row r="980">
-      <c r="G980" s="9"/>
+      <c r="C980" s="7"/>
     </row>
     <row r="981">
-      <c r="G981" s="9"/>
+      <c r="C981" s="7"/>
     </row>
     <row r="982">
-      <c r="G982" s="9"/>
+      <c r="C982" s="7"/>
     </row>
     <row r="983">
-      <c r="G983" s="9"/>
+      <c r="C983" s="7"/>
     </row>
     <row r="984">
-      <c r="G984" s="9"/>
+      <c r="C984" s="7"/>
     </row>
     <row r="985">
-      <c r="G985" s="9"/>
+      <c r="C985" s="7"/>
     </row>
     <row r="986">
-      <c r="G986" s="9"/>
+      <c r="C986" s="7"/>
     </row>
     <row r="987">
-      <c r="G987" s="9"/>
+      <c r="C987" s="7"/>
     </row>
     <row r="988">
-      <c r="G988" s="9"/>
+      <c r="C988" s="7"/>
     </row>
     <row r="989">
-      <c r="G989" s="9"/>
+      <c r="C989" s="7"/>
     </row>
     <row r="990">
-      <c r="G990" s="9"/>
+      <c r="C990" s="7"/>
     </row>
     <row r="991">
-      <c r="G991" s="9"/>
+      <c r="C991" s="7"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" horizontalCentered="1"/>

</xml_diff>